<commit_message>
Informe y modelo: sensibilidad del universo de commodities, desviaciones documentadas y preguntas para la defensa
- Tabla 3 ETF vs 5 ETF (control del sesgo de selección) en informe, Excel (09_Validacion) y run_all.py
- Sección 5: desviaciones de la regla con fecha y motivo (USO 14-sep, AFL/FRT 21-sep, Low-Vol 30-sep, petróleo 2-oct)
- Anexo B: preguntas anticipadas para la defensa; comisiones de StockTrak como costo operativo

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nexum_proyecto_final/modelo/Modelo_Nexum_v2.xlsx
+++ b/nexum_proyecto_final/modelo/Modelo_Nexum_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matiastorres/Desktop/Nexum_Proyecto_Final/modelo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1106CD7-3C83-7341-A425-FDEEB73A67DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D72E7677-56C0-294C-9815-523757F9BC1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_Indice" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="396">
   <si>
     <t>Nexum Financial Advisors — Modelo de inversión Familia Allende Cunich (v2)</t>
   </si>
@@ -1099,6 +1099,24 @@
   </si>
   <si>
     <t>Pesos iguales (1/6)</t>
+  </si>
+  <si>
+    <t>Sensibilidad al universo de commodities (control del sesgo de selección)</t>
+  </si>
+  <si>
+    <t>Cartera CAGR</t>
+  </si>
+  <si>
+    <t>P(3 objetivos) histórico</t>
+  </si>
+  <si>
+    <t>Peso BL recalibrado commodities</t>
+  </si>
+  <si>
+    <t>5 ETF (vigente: GLD, USO, DBA, SLV, CPER)</t>
+  </si>
+  <si>
+    <t>3 ETF (original: GLD, USO, DBA)</t>
   </si>
   <si>
     <t>Sesgos y limitaciones declarados</t>
@@ -1905,7 +1923,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="B2:O50"/>
+  <dimension ref="B2:O55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -2995,34 +3013,99 @@
         <v>352</v>
       </c>
     </row>
-    <row r="45" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B45" s="6" t="s">
+    <row r="45" spans="2:13" ht="42" x14ac:dyDescent="0.2">
+      <c r="B45" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C45" s="4" t="s">
         <v>353</v>
       </c>
+      <c r="D45" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>355</v>
+      </c>
     </row>
     <row r="46" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B46" s="6" t="s">
-        <v>354</v>
+      <c r="B46" s="26" t="s">
+        <v>356</v>
+      </c>
+      <c r="C46" s="27">
+        <v>9.9933608850413025E-2</v>
+      </c>
+      <c r="D46" s="35">
+        <v>0.84976461038245288</v>
+      </c>
+      <c r="E46" s="27">
+        <v>-0.20475279809972591</v>
+      </c>
+      <c r="F46" s="27">
+        <v>0.95955000000000001</v>
+      </c>
+      <c r="G46" s="27">
+        <v>6.5944584524457506E-2</v>
       </c>
     </row>
     <row r="47" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B47" s="6" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="48" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B48" s="6" t="s">
-        <v>356</v>
+      <c r="B47" s="26" t="s">
+        <v>357</v>
+      </c>
+      <c r="C47" s="27">
+        <v>9.7369402699195362E-2</v>
+      </c>
+      <c r="D47" s="35">
+        <v>0.83369296163192341</v>
+      </c>
+      <c r="E47" s="27">
+        <v>-0.20423033004416549</v>
+      </c>
+      <c r="F47" s="27">
+        <v>0.94769999999999999</v>
+      </c>
+      <c r="G47" s="27">
+        <v>0.1014848299326839</v>
       </c>
     </row>
     <row r="49" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B49" s="6" t="s">
-        <v>357</v>
+      <c r="B49" s="25" t="s">
+        <v>358</v>
       </c>
     </row>
     <row r="50" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B50" s="6" t="s">
-        <v>358</v>
+        <v>359</v>
+      </c>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B51" s="6" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B52" s="6" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B53" s="6" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B54" s="6" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B55" s="6" t="s">
+        <v>364</v>
       </c>
     </row>
   </sheetData>
@@ -3043,162 +3126,162 @@
   <sheetData>
     <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B5" s="4" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="48"/>
       <c r="B6" s="49" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="C6" s="49" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="D6" s="49" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A7" s="48"/>
       <c r="B7" s="49" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="C7" s="49" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="D7" s="49" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="48"/>
       <c r="B8" s="49" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="C8" s="49" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="D8" s="49" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A9" s="48"/>
       <c r="B9" s="49" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="C9" s="49" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="D9" s="49" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A10" s="48"/>
       <c r="B10" s="49" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="C10" s="49" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
       <c r="D10" s="49" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="48"/>
       <c r="B11" s="49" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="C11" s="49" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="D11" s="49" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="48"/>
       <c r="B12" s="49" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="C12" s="49" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="D12" s="49" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="48"/>
       <c r="B13" s="49" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="C13" s="49" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="D13" s="49" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="48"/>
       <c r="B14" s="49" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="C14" s="49" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="D14" s="49" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="48"/>
       <c r="B15" s="49" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="C15" s="49" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="D15" s="49" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="48"/>
       <c r="B16" s="49" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="C16" s="49" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
       <c r="D16" s="49" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="48"/>
       <c r="B17" s="49" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="C17" s="49" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="D17" s="49" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agregar análisis complementarios: contribución al riesgo, desempleo de Tomás y abanico del patrimonio
Rescatados del trabajo de Francisca (modelo_nexum/) y recalculados con el modelo oficial:
- Contribución al riesgo por activo (Python + fórmulas vivas en Excel, hoja 06)
- Montecarlo con desempleo persistente de Tomás, correlacionado con el mercado, y estrés de pérdida permanente
- Abanico del patrimonio real (percentiles 10-90), histórico y prospectivo
- Informe: nuevas figuras 3 y 7, tabla de capital humano; Excel: hojas 06 y 08 ampliadas

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nexum_proyecto_final/modelo/Modelo_Nexum_v2.xlsx
+++ b/nexum_proyecto_final/modelo/Modelo_Nexum_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matiastorres/Desktop/Nexum_Proyecto_Final/modelo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D72E7677-56C0-294C-9815-523757F9BC1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3036EDA6-0919-434E-85D8-62AC4DEB7EAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="415">
   <si>
     <t>Nexum Financial Advisors — Modelo de inversión Familia Allende Cunich (v2)</t>
   </si>
@@ -777,6 +777,21 @@
     <t>δ usado en Black-Litterman</t>
   </si>
   <si>
+    <t>Contribución al riesgo (pesos aprobados): w_i·(Σw)_i / w'Σw</t>
+  </si>
+  <si>
+    <t>Peso</t>
+  </si>
+  <si>
+    <t>Contribución marginal (Σw)_i</t>
+  </si>
+  <si>
+    <t>Contribución al riesgo (%)</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
     <t>Benchmark de política, métricas y tracking error</t>
   </si>
   <si>
@@ -786,9 +801,6 @@
     <t>Sleeve</t>
   </si>
   <si>
-    <t>Peso</t>
-  </si>
-  <si>
     <t>ICE U.S. Treasury 10-20 Year (TLH)</t>
   </si>
   <si>
@@ -943,6 +955,51 @@
   </si>
   <si>
     <t>Ambas</t>
+  </si>
+  <si>
+    <t>Capital humano: desempleo de Tomás (los aportes se cortan mientras está desempleado)</t>
+  </si>
+  <si>
+    <t>Escenario de empleo</t>
+  </si>
+  <si>
+    <t>Mercado</t>
+  </si>
+  <si>
+    <t>Sin desempleo (base)</t>
+  </si>
+  <si>
+    <t>Histórico</t>
+  </si>
+  <si>
+    <t>5% anual, independiente del mercado; reempleo en ~2 años</t>
+  </si>
+  <si>
+    <t>5% normal y 25% si la cartera cayó &gt;10% en 12 meses; reempleo ~2 años</t>
+  </si>
+  <si>
+    <t>10% normal y 40% si la cartera cayó &gt;10%; reempleo ~2 años</t>
+  </si>
+  <si>
+    <t>Estrés: 6% anual y pérdida PERMANENTE (sin reempleo)</t>
+  </si>
+  <si>
+    <t>Abanico del patrimonio real (USD de hoy) — percentiles al cierre de cada año</t>
+  </si>
+  <si>
+    <t>P10</t>
+  </si>
+  <si>
+    <t>P25</t>
+  </si>
+  <si>
+    <t>P50</t>
+  </si>
+  <si>
+    <t>P75</t>
+  </si>
+  <si>
+    <t>P90</t>
   </si>
   <si>
     <t>Validación: correcciones, robustez y prueba fuera de muestra</t>
@@ -1372,7 +1429,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1421,8 +1478,11 @@
     <xf numFmtId="10" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1934,61 +1994,61 @@
   <sheetData>
     <row r="2" spans="2:15" ht="18" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>300</v>
+        <v>319</v>
       </c>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B5" s="25" t="s">
-        <v>301</v>
+        <v>320</v>
       </c>
     </row>
     <row r="6" spans="2:15" ht="56" x14ac:dyDescent="0.2">
       <c r="B6" s="4" t="s">
-        <v>302</v>
+        <v>321</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>303</v>
+        <v>322</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>304</v>
+        <v>323</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>305</v>
+        <v>324</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>306</v>
+        <v>325</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>307</v>
+        <v>326</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>308</v>
+        <v>327</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>309</v>
+        <v>328</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>310</v>
+        <v>329</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>311</v>
+        <v>330</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>312</v>
+        <v>331</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>313</v>
+        <v>332</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>314</v>
+        <v>333</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>315</v>
+        <v>334</v>
       </c>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B7" s="26" t="s">
-        <v>316</v>
+        <v>335</v>
       </c>
       <c r="C7" s="31">
         <v>162</v>
@@ -2032,7 +2092,7 @@
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B8" s="26" t="s">
-        <v>317</v>
+        <v>336</v>
       </c>
       <c r="C8" s="31">
         <v>164</v>
@@ -2076,7 +2136,7 @@
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B9" s="26" t="s">
-        <v>318</v>
+        <v>337</v>
       </c>
       <c r="C9" s="31">
         <v>164</v>
@@ -2120,7 +2180,7 @@
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B10" s="26" t="s">
-        <v>319</v>
+        <v>338</v>
       </c>
       <c r="C10" s="31">
         <v>164</v>
@@ -2164,7 +2224,7 @@
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B12" s="25" t="s">
-        <v>320</v>
+        <v>339</v>
       </c>
     </row>
     <row r="13" spans="2:15" ht="28" x14ac:dyDescent="0.2">
@@ -2172,7 +2232,7 @@
         <v>93</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>321</v>
+        <v>340</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>167</v>
@@ -2187,18 +2247,18 @@
         <v>173</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>322</v>
+        <v>341</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>323</v>
+        <v>342</v>
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B14" s="26" t="s">
-        <v>324</v>
+        <v>343</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>325</v>
+        <v>344</v>
       </c>
       <c r="D14" s="27">
         <v>0.16184387692290139</v>
@@ -2221,10 +2281,10 @@
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B15" s="26" t="s">
-        <v>324</v>
+        <v>343</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>326</v>
+        <v>345</v>
       </c>
       <c r="D15" s="27">
         <v>0.17084228994553169</v>
@@ -2247,10 +2307,10 @@
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B16" s="26" t="s">
-        <v>324</v>
+        <v>343</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>327</v>
+        <v>346</v>
       </c>
       <c r="D16" s="27">
         <v>0.1766038087223831</v>
@@ -2273,10 +2333,10 @@
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B17" s="26" t="s">
-        <v>324</v>
+        <v>343</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>328</v>
+        <v>347</v>
       </c>
       <c r="D17" s="27">
         <v>0.16501389721692619</v>
@@ -2299,10 +2359,10 @@
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B18" s="26" t="s">
-        <v>324</v>
+        <v>343</v>
       </c>
       <c r="C18" s="26" t="s">
-        <v>329</v>
+        <v>348</v>
       </c>
       <c r="D18" s="27">
         <v>0.1350180936487877</v>
@@ -2325,10 +2385,10 @@
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B19" s="26" t="s">
-        <v>324</v>
+        <v>343</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>330</v>
+        <v>349</v>
       </c>
       <c r="D19" s="27">
         <v>0.12811353145566501</v>
@@ -2351,10 +2411,10 @@
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B20" s="26" t="s">
-        <v>324</v>
+        <v>343</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="D20" s="27">
         <v>0.16629562491536351</v>
@@ -2377,10 +2437,10 @@
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B21" s="26" t="s">
-        <v>324</v>
+        <v>343</v>
       </c>
       <c r="C21" s="26" t="s">
-        <v>332</v>
+        <v>351</v>
       </c>
       <c r="D21" s="27">
         <v>0.18608357972450729</v>
@@ -2406,7 +2466,7 @@
         <v>105</v>
       </c>
       <c r="C22" s="26" t="s">
-        <v>325</v>
+        <v>344</v>
       </c>
       <c r="D22" s="27">
         <v>0.1071607336590132</v>
@@ -2432,7 +2492,7 @@
         <v>105</v>
       </c>
       <c r="C23" s="26" t="s">
-        <v>329</v>
+        <v>348</v>
       </c>
       <c r="D23" s="27">
         <v>0.1049851840260618</v>
@@ -2458,7 +2518,7 @@
         <v>105</v>
       </c>
       <c r="C24" s="26" t="s">
-        <v>330</v>
+        <v>349</v>
       </c>
       <c r="D24" s="27">
         <v>0.10992134335539069</v>
@@ -2484,7 +2544,7 @@
         <v>105</v>
       </c>
       <c r="C25" s="26" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="D25" s="27">
         <v>0.1065487985195943</v>
@@ -2510,7 +2570,7 @@
         <v>105</v>
       </c>
       <c r="C26" s="26" t="s">
-        <v>332</v>
+        <v>351</v>
       </c>
       <c r="D26" s="27">
         <v>0.10252224545788401</v>
@@ -2533,10 +2593,10 @@
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B27" s="26" t="s">
-        <v>333</v>
+        <v>352</v>
       </c>
       <c r="C27" s="26" t="s">
-        <v>334</v>
+        <v>353</v>
       </c>
       <c r="D27" s="27">
         <v>7.9459140073918397E-2</v>
@@ -2559,10 +2619,10 @@
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B28" s="26" t="s">
-        <v>333</v>
+        <v>352</v>
       </c>
       <c r="C28" s="26" t="s">
-        <v>335</v>
+        <v>354</v>
       </c>
       <c r="D28" s="27">
         <v>4.0834405761133799E-2</v>
@@ -2585,10 +2645,10 @@
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B29" s="26" t="s">
-        <v>333</v>
+        <v>352</v>
       </c>
       <c r="C29" s="26" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="D29" s="27">
         <v>5.2424311770700997E-2</v>
@@ -2611,10 +2671,10 @@
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B30" s="26" t="s">
-        <v>333</v>
+        <v>352</v>
       </c>
       <c r="C30" s="26" t="s">
-        <v>337</v>
+        <v>356</v>
       </c>
       <c r="D30" s="27">
         <v>4.32542159789195E-2</v>
@@ -2637,10 +2697,10 @@
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B31" s="26" t="s">
-        <v>333</v>
+        <v>352</v>
       </c>
       <c r="C31" s="26" t="s">
-        <v>338</v>
+        <v>357</v>
       </c>
       <c r="D31" s="27">
         <v>8.0896159321954597E-2</v>
@@ -2663,7 +2723,7 @@
     </row>
     <row r="33" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B33" s="25" t="s">
-        <v>339</v>
+        <v>358</v>
       </c>
     </row>
     <row r="34" spans="2:13" x14ac:dyDescent="0.2">
@@ -2671,7 +2731,7 @@
         <v>103</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>167</v>
@@ -2686,30 +2746,30 @@
         <v>173</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>340</v>
+        <v>359</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>341</v>
+        <v>360</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>342</v>
+        <v>361</v>
       </c>
       <c r="K34" s="4" t="s">
-        <v>343</v>
+        <v>362</v>
       </c>
       <c r="L34" s="4" t="s">
-        <v>344</v>
+        <v>363</v>
       </c>
       <c r="M34" s="4" t="s">
-        <v>345</v>
+        <v>364</v>
       </c>
     </row>
     <row r="35" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B35" s="26" t="s">
-        <v>346</v>
+        <v>365</v>
       </c>
       <c r="C35" s="26" t="s">
-        <v>347</v>
+        <v>366</v>
       </c>
       <c r="D35" s="27">
         <v>0.1056683972588288</v>
@@ -2744,10 +2804,10 @@
     </row>
     <row r="36" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B36" s="26" t="s">
-        <v>346</v>
+        <v>365</v>
       </c>
       <c r="C36" s="26" t="s">
-        <v>348</v>
+        <v>367</v>
       </c>
       <c r="D36" s="27">
         <v>7.4513279706229119E-2</v>
@@ -2782,10 +2842,10 @@
     </row>
     <row r="37" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B37" s="26" t="s">
-        <v>349</v>
+        <v>368</v>
       </c>
       <c r="C37" s="26" t="s">
-        <v>347</v>
+        <v>366</v>
       </c>
       <c r="D37" s="27">
         <v>0.1201605662353227</v>
@@ -2820,10 +2880,10 @@
     </row>
     <row r="38" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B38" s="26" t="s">
-        <v>349</v>
+        <v>368</v>
       </c>
       <c r="C38" s="26" t="s">
-        <v>348</v>
+        <v>367</v>
       </c>
       <c r="D38" s="27">
         <v>0.1107305716741742</v>
@@ -2858,10 +2918,10 @@
     </row>
     <row r="39" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B39" s="26" t="s">
-        <v>350</v>
+        <v>369</v>
       </c>
       <c r="C39" s="26" t="s">
-        <v>347</v>
+        <v>366</v>
       </c>
       <c r="D39" s="27">
         <v>0.10761655035187891</v>
@@ -2896,10 +2956,10 @@
     </row>
     <row r="40" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B40" s="26" t="s">
-        <v>350</v>
+        <v>369</v>
       </c>
       <c r="C40" s="26" t="s">
-        <v>348</v>
+        <v>367</v>
       </c>
       <c r="D40" s="27">
         <v>9.1923869622193344E-2</v>
@@ -2934,10 +2994,10 @@
     </row>
     <row r="41" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B41" s="26" t="s">
-        <v>351</v>
+        <v>370</v>
       </c>
       <c r="C41" s="26" t="s">
-        <v>347</v>
+        <v>366</v>
       </c>
       <c r="D41" s="27">
         <v>9.5147502223999592E-2</v>
@@ -2972,10 +3032,10 @@
     </row>
     <row r="42" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B42" s="26" t="s">
-        <v>351</v>
+        <v>370</v>
       </c>
       <c r="C42" s="26" t="s">
-        <v>348</v>
+        <v>367</v>
       </c>
       <c r="D42" s="27">
         <v>9.3137149390628116E-2</v>
@@ -3010,7 +3070,7 @@
     </row>
     <row r="44" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B44" s="25" t="s">
-        <v>352</v>
+        <v>371</v>
       </c>
     </row>
     <row r="45" spans="2:13" ht="42" x14ac:dyDescent="0.2">
@@ -3018,24 +3078,24 @@
         <v>97</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>353</v>
+        <v>372</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>308</v>
+        <v>327</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>309</v>
+        <v>328</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>354</v>
+        <v>373</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>355</v>
+        <v>374</v>
       </c>
     </row>
     <row r="46" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B46" s="26" t="s">
-        <v>356</v>
+        <v>375</v>
       </c>
       <c r="C46" s="27">
         <v>9.9933608850413025E-2</v>
@@ -3055,7 +3115,7 @@
     </row>
     <row r="47" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B47" s="26" t="s">
-        <v>357</v>
+        <v>376</v>
       </c>
       <c r="C47" s="27">
         <v>9.7369402699195362E-2</v>
@@ -3075,37 +3135,37 @@
     </row>
     <row r="49" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B49" s="25" t="s">
-        <v>358</v>
+        <v>377</v>
       </c>
     </row>
     <row r="50" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B50" s="6" t="s">
-        <v>359</v>
+        <v>378</v>
       </c>
     </row>
     <row r="51" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B51" s="6" t="s">
-        <v>360</v>
+        <v>379</v>
       </c>
     </row>
     <row r="52" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B52" s="6" t="s">
-        <v>361</v>
+        <v>380</v>
       </c>
     </row>
     <row r="53" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B53" s="6" t="s">
-        <v>362</v>
+        <v>381</v>
       </c>
     </row>
     <row r="54" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B54" s="6" t="s">
-        <v>363</v>
+        <v>382</v>
       </c>
     </row>
     <row r="55" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B55" s="6" t="s">
-        <v>364</v>
+        <v>383</v>
       </c>
     </row>
   </sheetData>
@@ -3126,162 +3186,162 @@
   <sheetData>
     <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>365</v>
+        <v>384</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B5" s="4" t="s">
-        <v>366</v>
+        <v>385</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>367</v>
+        <v>386</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>368</v>
+        <v>387</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="48"/>
-      <c r="B6" s="49" t="s">
-        <v>369</v>
-      </c>
-      <c r="C6" s="49" t="s">
-        <v>370</v>
-      </c>
-      <c r="D6" s="49" t="s">
-        <v>371</v>
+      <c r="A6" s="51"/>
+      <c r="B6" s="52" t="s">
+        <v>388</v>
+      </c>
+      <c r="C6" s="52" t="s">
+        <v>389</v>
+      </c>
+      <c r="D6" s="52" t="s">
+        <v>390</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="28" x14ac:dyDescent="0.2">
-      <c r="A7" s="48"/>
-      <c r="B7" s="49" t="s">
-        <v>369</v>
-      </c>
-      <c r="C7" s="49" t="s">
-        <v>372</v>
-      </c>
-      <c r="D7" s="49" t="s">
-        <v>373</v>
+      <c r="A7" s="51"/>
+      <c r="B7" s="52" t="s">
+        <v>388</v>
+      </c>
+      <c r="C7" s="52" t="s">
+        <v>391</v>
+      </c>
+      <c r="D7" s="52" t="s">
+        <v>392</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="48"/>
-      <c r="B8" s="49" t="s">
-        <v>369</v>
-      </c>
-      <c r="C8" s="49" t="s">
-        <v>374</v>
-      </c>
-      <c r="D8" s="49" t="s">
-        <v>375</v>
+      <c r="A8" s="51"/>
+      <c r="B8" s="52" t="s">
+        <v>388</v>
+      </c>
+      <c r="C8" s="52" t="s">
+        <v>393</v>
+      </c>
+      <c r="D8" s="52" t="s">
+        <v>394</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="28" x14ac:dyDescent="0.2">
-      <c r="A9" s="48"/>
-      <c r="B9" s="49" t="s">
-        <v>369</v>
-      </c>
-      <c r="C9" s="49" t="s">
-        <v>376</v>
-      </c>
-      <c r="D9" s="49" t="s">
-        <v>377</v>
+      <c r="A9" s="51"/>
+      <c r="B9" s="52" t="s">
+        <v>388</v>
+      </c>
+      <c r="C9" s="52" t="s">
+        <v>395</v>
+      </c>
+      <c r="D9" s="52" t="s">
+        <v>396</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="28" x14ac:dyDescent="0.2">
-      <c r="A10" s="48"/>
-      <c r="B10" s="49" t="s">
-        <v>369</v>
-      </c>
-      <c r="C10" s="49" t="s">
-        <v>378</v>
-      </c>
-      <c r="D10" s="49" t="s">
-        <v>379</v>
+      <c r="A10" s="51"/>
+      <c r="B10" s="52" t="s">
+        <v>388</v>
+      </c>
+      <c r="C10" s="52" t="s">
+        <v>397</v>
+      </c>
+      <c r="D10" s="52" t="s">
+        <v>398</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="48"/>
-      <c r="B11" s="49" t="s">
-        <v>380</v>
-      </c>
-      <c r="C11" s="49" t="s">
-        <v>381</v>
-      </c>
-      <c r="D11" s="49" t="s">
-        <v>382</v>
+      <c r="A11" s="51"/>
+      <c r="B11" s="52" t="s">
+        <v>399</v>
+      </c>
+      <c r="C11" s="52" t="s">
+        <v>400</v>
+      </c>
+      <c r="D11" s="52" t="s">
+        <v>401</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="48"/>
-      <c r="B12" s="49" t="s">
-        <v>380</v>
-      </c>
-      <c r="C12" s="49" t="s">
-        <v>383</v>
-      </c>
-      <c r="D12" s="49" t="s">
-        <v>384</v>
+      <c r="A12" s="51"/>
+      <c r="B12" s="52" t="s">
+        <v>399</v>
+      </c>
+      <c r="C12" s="52" t="s">
+        <v>402</v>
+      </c>
+      <c r="D12" s="52" t="s">
+        <v>403</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="48"/>
-      <c r="B13" s="49" t="s">
-        <v>380</v>
-      </c>
-      <c r="C13" s="49" t="s">
-        <v>385</v>
-      </c>
-      <c r="D13" s="49" t="s">
-        <v>386</v>
+      <c r="A13" s="51"/>
+      <c r="B13" s="52" t="s">
+        <v>399</v>
+      </c>
+      <c r="C13" s="52" t="s">
+        <v>404</v>
+      </c>
+      <c r="D13" s="52" t="s">
+        <v>405</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="48"/>
-      <c r="B14" s="49" t="s">
-        <v>380</v>
-      </c>
-      <c r="C14" s="49" t="s">
-        <v>387</v>
-      </c>
-      <c r="D14" s="49" t="s">
-        <v>388</v>
+      <c r="A14" s="51"/>
+      <c r="B14" s="52" t="s">
+        <v>399</v>
+      </c>
+      <c r="C14" s="52" t="s">
+        <v>406</v>
+      </c>
+      <c r="D14" s="52" t="s">
+        <v>407</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="48"/>
-      <c r="B15" s="49" t="s">
-        <v>389</v>
-      </c>
-      <c r="C15" s="49" t="s">
-        <v>390</v>
-      </c>
-      <c r="D15" s="49" t="s">
-        <v>391</v>
+      <c r="A15" s="51"/>
+      <c r="B15" s="52" t="s">
+        <v>408</v>
+      </c>
+      <c r="C15" s="52" t="s">
+        <v>409</v>
+      </c>
+      <c r="D15" s="52" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="48"/>
-      <c r="B16" s="49" t="s">
-        <v>389</v>
-      </c>
-      <c r="C16" s="49" t="s">
-        <v>392</v>
-      </c>
-      <c r="D16" s="49" t="s">
-        <v>393</v>
+      <c r="A16" s="51"/>
+      <c r="B16" s="52" t="s">
+        <v>408</v>
+      </c>
+      <c r="C16" s="52" t="s">
+        <v>411</v>
+      </c>
+      <c r="D16" s="52" t="s">
+        <v>412</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="48"/>
-      <c r="B17" s="49" t="s">
-        <v>389</v>
-      </c>
-      <c r="C17" s="49" t="s">
-        <v>394</v>
-      </c>
-      <c r="D17" s="49" t="s">
-        <v>395</v>
+      <c r="A17" s="51"/>
+      <c r="B17" s="52" t="s">
+        <v>408</v>
+      </c>
+      <c r="C17" s="52" t="s">
+        <v>413</v>
+      </c>
+      <c r="D17" s="52" t="s">
+        <v>414</v>
       </c>
     </row>
   </sheetData>
@@ -13719,7 +13779,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="B2:K52"/>
+  <dimension ref="B2:K62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -14314,7 +14374,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B49" s="4" t="s">
         <v>156</v>
       </c>
@@ -14322,7 +14382,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B50" s="26" t="s">
         <v>241</v>
       </c>
@@ -14330,7 +14390,7 @@
         <v>6.6789022507229836</v>
       </c>
     </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B51" s="26" t="s">
         <v>242</v>
       </c>
@@ -14338,12 +14398,137 @@
         <v>3.3358139907403839</v>
       </c>
     </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B52" s="26" t="s">
         <v>243</v>
       </c>
       <c r="C52" s="35">
         <v>2.5</v>
+      </c>
+    </row>
+    <row r="54" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B54" s="25" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="55" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B55" s="46" t="s">
+        <v>116</v>
+      </c>
+      <c r="C55" s="46" t="s">
+        <v>245</v>
+      </c>
+      <c r="D55" s="46" t="s">
+        <v>246</v>
+      </c>
+      <c r="E55" s="46" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="56" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B56" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C56" s="43">
+        <f>'05_Markowitz'!F6</f>
+        <v>0.37890000000000001</v>
+      </c>
+      <c r="D56" s="47">
+        <f t="array" ref="D56:D61">MMULT('05_Markowitz'!C15:H20,'05_Markowitz'!F6:F11)</f>
+        <v>1.2844708860157737E-2</v>
+      </c>
+      <c r="E56" s="22">
+        <f t="shared" ref="E56:E61" si="3">C56*D56/SUMPRODUCT($C$56:$C$61,$D$56:$D$61)</f>
+        <v>0.49526431319301806</v>
+      </c>
+    </row>
+    <row r="57" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B57" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="C57" s="43">
+        <f>'05_Markowitz'!F7</f>
+        <v>0.16869999999999999</v>
+      </c>
+      <c r="D57" s="47">
+        <v>4.3070105897552264E-3</v>
+      </c>
+      <c r="E57" s="22">
+        <f t="shared" si="3"/>
+        <v>7.3939955949257077E-2</v>
+      </c>
+    </row>
+    <row r="58" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B58" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="C58" s="43">
+        <f>'05_Markowitz'!F8</f>
+        <v>0.14599999999999999</v>
+      </c>
+      <c r="D58" s="47">
+        <v>8.2847754186396554E-3</v>
+      </c>
+      <c r="E58" s="22">
+        <f t="shared" si="3"/>
+        <v>0.12308971363223541</v>
+      </c>
+    </row>
+    <row r="59" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B59" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C59" s="43">
+        <f>'05_Markowitz'!F9</f>
+        <v>6.1100000000000002E-2</v>
+      </c>
+      <c r="D59" s="47">
+        <v>4.1718877011711194E-3</v>
+      </c>
+      <c r="E59" s="22">
+        <f t="shared" si="3"/>
+        <v>2.5939522972807057E-2</v>
+      </c>
+    </row>
+    <row r="60" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B60" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C60" s="43">
+        <f>'05_Markowitz'!F10</f>
+        <v>7.0599999999999996E-2</v>
+      </c>
+      <c r="D60" s="47">
+        <v>1.6572798184914427E-2</v>
+      </c>
+      <c r="E60" s="22">
+        <f t="shared" si="3"/>
+        <v>0.11906625889776498</v>
+      </c>
+    </row>
+    <row r="61" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B61" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C61" s="43">
+        <f>'05_Markowitz'!F11</f>
+        <v>0.17460000000000001</v>
+      </c>
+      <c r="D61" s="47">
+        <v>9.1570540251548448E-3</v>
+      </c>
+      <c r="E61" s="22">
+        <f t="shared" si="3"/>
+        <v>0.16270023535491743</v>
+      </c>
+    </row>
+    <row r="62" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B62" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="E62" s="22">
+        <f>SUM(E56:E61)</f>
+        <v>1.0000000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -14365,20 +14550,20 @@
   <sheetData>
     <row r="2" spans="2:16" ht="18" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B5" s="4" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>166</v>
@@ -14388,7 +14573,7 @@
       <c r="B6" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="C6" s="46">
+      <c r="C6" s="48">
         <v>0.37890000000000001</v>
       </c>
       <c r="D6" s="6" t="s">
@@ -14399,68 +14584,68 @@
       <c r="B7" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="C7" s="46">
+      <c r="C7" s="48">
         <v>0.16869999999999999</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B8" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="C8" s="46">
+      <c r="C8" s="48">
         <v>0.14599999999999999</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="9" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B9" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="C9" s="46">
+      <c r="C9" s="48">
         <v>6.1100000000000002E-2</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="10" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B10" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="C10" s="46">
+      <c r="C10" s="48">
         <v>7.0599999999999996E-2</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="11" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B11" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="C11" s="46">
+      <c r="C11" s="48">
         <v>0.17460000000000001</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="13" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B13" s="25" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="14" spans="2:16" ht="28" x14ac:dyDescent="0.2">
       <c r="B14" s="4" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>167</v>
@@ -14475,7 +14660,7 @@
         <v>170</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="I14" s="4" t="s">
         <v>171</v>
@@ -14487,7 +14672,7 @@
         <v>173</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="M14" s="4" t="s">
         <v>174</v>
@@ -14504,10 +14689,10 @@
     </row>
     <row r="15" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B15" s="26" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="D15" s="27">
         <v>9.9022250785216759E-2</v>
@@ -14551,10 +14736,10 @@
     </row>
     <row r="16" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B16" s="26" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="D16" s="27">
         <v>9.4618530441715754E-2</v>
@@ -14596,10 +14781,10 @@
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B17" s="26" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="D17" s="27">
         <v>0.1265263686562654</v>
@@ -14643,7 +14828,7 @@
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B18" s="26" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="C18" s="26" t="s">
         <v>200</v>
@@ -14690,10 +14875,10 @@
     </row>
     <row r="19" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B19" s="26" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="D19" s="27">
         <v>9.9933608850413025E-2</v>
@@ -14733,10 +14918,10 @@
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B20" s="26" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="D20" s="27">
         <v>0.1220358386781133</v>
@@ -14776,7 +14961,7 @@
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B21" s="26" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="C21" s="26" t="s">
         <v>200</v>
@@ -14819,7 +15004,7 @@
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B24" s="25" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.2">
@@ -14832,7 +15017,7 @@
     </row>
     <row r="26" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B26" s="26" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="C26" s="27">
         <v>2.0174150134109739E-2</v>
@@ -14840,7 +15025,7 @@
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B27" s="26" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="C27" s="27">
         <v>2.419747732560756E-2</v>
@@ -14872,7 +15057,7 @@
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B31" s="26" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="C31" s="27">
         <v>0.04</v>
@@ -14880,7 +15065,7 @@
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B32" s="26" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C32" s="27">
         <v>0</v>
@@ -14888,7 +15073,7 @@
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B33" s="26" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="C33" s="27">
         <v>0</v>
@@ -14896,7 +15081,7 @@
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B34" s="26" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="C34" s="27">
         <v>0</v>
@@ -14904,7 +15089,7 @@
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B35" s="26" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="C35" s="27">
         <v>0.17516200585592129</v>
@@ -14912,7 +15097,7 @@
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B36" s="26" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C36" s="27">
         <v>0.1897073484073088</v>
@@ -14920,7 +15105,7 @@
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B37" s="26" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="C37" s="27">
         <v>4.4320618292240009E-2</v>
@@ -14933,7 +15118,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="B2:Q21"/>
+  <dimension ref="B2:Q91"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -14945,12 +15130,12 @@
   <sheetData>
     <row r="2" spans="2:17" ht="18" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
     <row r="3" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5" spans="2:17" ht="28" x14ac:dyDescent="0.2">
@@ -14961,71 +15146,71 @@
         <v>131</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="O5" s="4" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="P5" s="4" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="Q5" s="4" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
     </row>
     <row r="6" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B6" s="26" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>291</v>
-      </c>
-      <c r="E6" s="47">
+        <v>295</v>
+      </c>
+      <c r="E6" s="49">
         <v>7.8368404371000455E-2</v>
       </c>
-      <c r="F6" s="47">
+      <c r="F6" s="49">
         <v>1</v>
       </c>
-      <c r="G6" s="47">
+      <c r="G6" s="49">
         <v>0.98134999999999994</v>
       </c>
-      <c r="H6" s="47">
+      <c r="H6" s="49">
         <v>0.95955000000000001</v>
       </c>
-      <c r="I6" s="47">
+      <c r="I6" s="49">
         <v>0.95955000000000001</v>
       </c>
       <c r="J6" s="32">
@@ -15043,10 +15228,10 @@
       <c r="N6" s="32">
         <v>5448079.025805857</v>
       </c>
-      <c r="O6" s="47">
+      <c r="O6" s="49">
         <v>-0.24062233506065539</v>
       </c>
-      <c r="P6" s="47">
+      <c r="P6" s="49">
         <v>-0.36194798736869083</v>
       </c>
       <c r="Q6" s="26" t="s">
@@ -15055,27 +15240,27 @@
     </row>
     <row r="7" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B7" s="26" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="D7" s="26" t="s">
         <v>158</v>
       </c>
-      <c r="E7" s="47">
+      <c r="E7" s="49">
         <v>7.8368404371000455E-2</v>
       </c>
-      <c r="F7" s="47">
+      <c r="F7" s="49">
         <v>1</v>
       </c>
-      <c r="G7" s="47">
+      <c r="G7" s="49">
         <v>0.91949999999999998</v>
       </c>
-      <c r="H7" s="47">
+      <c r="H7" s="49">
         <v>0.89644999999999997</v>
       </c>
-      <c r="I7" s="47">
+      <c r="I7" s="49">
         <v>0.89644999999999997</v>
       </c>
       <c r="J7" s="32">
@@ -15093,10 +15278,10 @@
       <c r="N7" s="32">
         <v>119629.0907291305</v>
       </c>
-      <c r="O7" s="47">
+      <c r="O7" s="49">
         <v>-0.24062233506065539</v>
       </c>
-      <c r="P7" s="47">
+      <c r="P7" s="49">
         <v>-0.36194798736869083</v>
       </c>
       <c r="Q7" s="26" t="s">
@@ -15105,27 +15290,27 @@
     </row>
     <row r="8" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B8" s="26" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>291</v>
-      </c>
-      <c r="E8" s="47">
+        <v>295</v>
+      </c>
+      <c r="E8" s="49">
         <v>4.5786922986983607E-2</v>
       </c>
-      <c r="F8" s="47">
+      <c r="F8" s="49">
         <v>1</v>
       </c>
-      <c r="G8" s="47">
+      <c r="G8" s="49">
         <v>0.71299999999999997</v>
       </c>
-      <c r="H8" s="47">
+      <c r="H8" s="49">
         <v>0.46529999999999999</v>
       </c>
-      <c r="I8" s="47">
+      <c r="I8" s="49">
         <v>0.46529999999999999</v>
       </c>
       <c r="J8" s="32">
@@ -15143,10 +15328,10 @@
       <c r="N8" s="32">
         <v>414317.88061139139</v>
       </c>
-      <c r="O8" s="47">
+      <c r="O8" s="49">
         <v>-0.30455108566934141</v>
       </c>
-      <c r="P8" s="47">
+      <c r="P8" s="49">
         <v>-0.46649885395855339</v>
       </c>
       <c r="Q8" s="26" t="s">
@@ -15155,27 +15340,27 @@
     </row>
     <row r="9" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B9" s="26" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="D9" s="26" t="s">
         <v>158</v>
       </c>
-      <c r="E9" s="47">
+      <c r="E9" s="49">
         <v>4.5786922986983607E-2</v>
       </c>
-      <c r="F9" s="47">
+      <c r="F9" s="49">
         <v>0.999</v>
       </c>
-      <c r="G9" s="47">
+      <c r="G9" s="49">
         <v>0.64510000000000001</v>
       </c>
-      <c r="H9" s="47">
+      <c r="H9" s="49">
         <v>0.45340000000000003</v>
       </c>
-      <c r="I9" s="47">
+      <c r="I9" s="49">
         <v>0.45340000000000003</v>
       </c>
       <c r="J9" s="32">
@@ -15193,10 +15378,10 @@
       <c r="N9" s="32">
         <v>9146.1088127118928</v>
       </c>
-      <c r="O9" s="47">
+      <c r="O9" s="49">
         <v>-0.30455108566934141</v>
       </c>
-      <c r="P9" s="47">
+      <c r="P9" s="49">
         <v>-0.46649885395855339</v>
       </c>
       <c r="Q9" s="26" t="s">
@@ -15205,27 +15390,27 @@
     </row>
     <row r="10" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B10" s="26" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="D10" s="26" t="s">
-        <v>291</v>
-      </c>
-      <c r="E10" s="47">
+        <v>295</v>
+      </c>
+      <c r="E10" s="49">
         <v>0.10003513595893419</v>
       </c>
-      <c r="F10" s="47">
+      <c r="F10" s="49">
         <v>1</v>
       </c>
-      <c r="G10" s="47">
+      <c r="G10" s="49">
         <v>0.99285000000000001</v>
       </c>
-      <c r="H10" s="47">
+      <c r="H10" s="49">
         <v>0.98809999999999998</v>
       </c>
-      <c r="I10" s="47">
+      <c r="I10" s="49">
         <v>0.98809999999999998</v>
       </c>
       <c r="J10" s="32">
@@ -15243,10 +15428,10 @@
       <c r="N10" s="32">
         <v>17614178.04023492</v>
       </c>
-      <c r="O10" s="47">
+      <c r="O10" s="49">
         <v>-0.28654946095590711</v>
       </c>
-      <c r="P10" s="47">
+      <c r="P10" s="49">
         <v>-0.4229171876989673</v>
       </c>
       <c r="Q10" s="26" t="s">
@@ -15255,27 +15440,27 @@
     </row>
     <row r="11" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B11" s="26" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="D11" s="26" t="s">
         <v>158</v>
       </c>
-      <c r="E11" s="47">
+      <c r="E11" s="49">
         <v>0.10003513595893419</v>
       </c>
-      <c r="F11" s="47">
+      <c r="F11" s="49">
         <v>0.99995000000000001</v>
       </c>
-      <c r="G11" s="47">
+      <c r="G11" s="49">
         <v>0.96950000000000003</v>
       </c>
-      <c r="H11" s="47">
+      <c r="H11" s="49">
         <v>0.96355000000000002</v>
       </c>
-      <c r="I11" s="47">
+      <c r="I11" s="49">
         <v>0.96355000000000002</v>
       </c>
       <c r="J11" s="32">
@@ -15293,10 +15478,10 @@
       <c r="N11" s="32">
         <v>338927.80074492359</v>
       </c>
-      <c r="O11" s="47">
+      <c r="O11" s="49">
         <v>-0.28654946095590711</v>
       </c>
-      <c r="P11" s="47">
+      <c r="P11" s="49">
         <v>-0.4229171876989673</v>
       </c>
       <c r="Q11" s="26" t="s">
@@ -15305,27 +15490,27 @@
     </row>
     <row r="12" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B12" s="26" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>291</v>
-      </c>
-      <c r="E12" s="47">
+        <v>295</v>
+      </c>
+      <c r="E12" s="49">
         <v>4.3773078585227942E-2</v>
       </c>
-      <c r="F12" s="47">
+      <c r="F12" s="49">
         <v>1</v>
       </c>
-      <c r="G12" s="47">
+      <c r="G12" s="49">
         <v>0.63580000000000003</v>
       </c>
-      <c r="H12" s="47">
+      <c r="H12" s="49">
         <v>0.42409999999999998</v>
       </c>
-      <c r="I12" s="47">
+      <c r="I12" s="49">
         <v>0.42409999999999998</v>
       </c>
       <c r="J12" s="32">
@@ -15343,10 +15528,10 @@
       <c r="N12" s="32">
         <v>290421.97347554541</v>
       </c>
-      <c r="O12" s="47">
+      <c r="O12" s="49">
         <v>-0.39765385285037019</v>
       </c>
-      <c r="P12" s="47">
+      <c r="P12" s="49">
         <v>-0.59753696749611229</v>
       </c>
       <c r="Q12" s="26" t="s">
@@ -15355,27 +15540,27 @@
     </row>
     <row r="13" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B13" s="26" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="D13" s="26" t="s">
         <v>158</v>
       </c>
-      <c r="E13" s="47">
+      <c r="E13" s="49">
         <v>4.3773078585227942E-2</v>
       </c>
-      <c r="F13" s="47">
+      <c r="F13" s="49">
         <v>0.99639999999999995</v>
       </c>
-      <c r="G13" s="47">
+      <c r="G13" s="49">
         <v>0.57220000000000004</v>
       </c>
-      <c r="H13" s="47">
+      <c r="H13" s="49">
         <v>0.3836</v>
       </c>
-      <c r="I13" s="47">
+      <c r="I13" s="49">
         <v>0.3836</v>
       </c>
       <c r="J13" s="32">
@@ -15393,10 +15578,10 @@
       <c r="N13" s="32">
         <v>3866.547472223303</v>
       </c>
-      <c r="O13" s="47">
+      <c r="O13" s="49">
         <v>-0.39765385285037019</v>
       </c>
-      <c r="P13" s="47">
+      <c r="P13" s="49">
         <v>-0.59753696749611229</v>
       </c>
       <c r="Q13" s="26" t="s">
@@ -15405,92 +15590,2306 @@
     </row>
     <row r="16" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B16" s="25" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6" ht="42" x14ac:dyDescent="0.2">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" ht="42" x14ac:dyDescent="0.2">
       <c r="B17" s="4" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.2">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="26" t="s">
+        <v>300</v>
+      </c>
+      <c r="C18" s="49">
+        <v>1</v>
+      </c>
+      <c r="D18" s="49">
+        <v>0.71299999999999997</v>
+      </c>
+      <c r="E18" s="49">
+        <v>0.46529999999999999</v>
+      </c>
+      <c r="F18" s="49">
+        <v>0.46529999999999999</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B19" s="26" t="s">
+        <v>301</v>
+      </c>
+      <c r="C19" s="49">
+        <v>1</v>
+      </c>
+      <c r="D19" s="49">
+        <v>0.71299999999999997</v>
+      </c>
+      <c r="E19" s="49">
+        <v>0.57620000000000005</v>
+      </c>
+      <c r="F19" s="49">
+        <v>0.57620000000000005</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B20" s="26" t="s">
+        <v>302</v>
+      </c>
+      <c r="C20" s="49">
+        <v>1</v>
+      </c>
+      <c r="D20" s="49">
+        <v>0.86980000000000002</v>
+      </c>
+      <c r="E20" s="49">
+        <v>0.62109999999999999</v>
+      </c>
+      <c r="F20" s="49">
+        <v>0.62109999999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B21" s="26" t="s">
+        <v>303</v>
+      </c>
+      <c r="C21" s="49">
+        <v>1</v>
+      </c>
+      <c r="D21" s="49">
+        <v>0.86980000000000002</v>
+      </c>
+      <c r="E21" s="49">
+        <v>0.74829999999999997</v>
+      </c>
+      <c r="F21" s="49">
+        <v>0.74829999999999997</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B24" s="25" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="B25" s="4" t="s">
+        <v>305</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B26" s="26" t="s">
+        <v>307</v>
+      </c>
+      <c r="C26" s="26" t="s">
+        <v>308</v>
+      </c>
+      <c r="D26" s="49">
+        <v>1</v>
+      </c>
+      <c r="E26" s="49">
+        <v>0.98134999999999994</v>
+      </c>
+      <c r="F26" s="49">
+        <v>0.95955000000000001</v>
+      </c>
+      <c r="G26" s="49">
+        <v>0.95955000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B27" s="26" t="s">
+        <v>307</v>
+      </c>
+      <c r="C27" s="26" t="s">
         <v>296</v>
       </c>
-      <c r="C18" s="47">
+      <c r="D27" s="49">
         <v>1</v>
       </c>
-      <c r="D18" s="47">
+      <c r="E27" s="49">
         <v>0.71299999999999997</v>
       </c>
-      <c r="E18" s="47">
+      <c r="F27" s="49">
         <v>0.46529999999999999</v>
       </c>
-      <c r="F18" s="47">
+      <c r="G27" s="49">
         <v>0.46529999999999999</v>
       </c>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B19" s="26" t="s">
-        <v>297</v>
-      </c>
-      <c r="C19" s="47">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B28" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="C28" s="26" t="s">
+        <v>308</v>
+      </c>
+      <c r="D28" s="49">
         <v>1</v>
       </c>
-      <c r="D19" s="47">
-        <v>0.71299999999999997</v>
-      </c>
-      <c r="E19" s="47">
-        <v>0.57620000000000005</v>
-      </c>
-      <c r="F19" s="47">
-        <v>0.57620000000000005</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B20" s="26" t="s">
-        <v>298</v>
-      </c>
-      <c r="C20" s="47">
+      <c r="E28" s="49">
+        <v>0.97435000000000005</v>
+      </c>
+      <c r="F28" s="49">
+        <v>0.94750000000000001</v>
+      </c>
+      <c r="G28" s="49">
+        <v>0.94750000000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B29" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="C29" s="26" t="s">
+        <v>296</v>
+      </c>
+      <c r="D29" s="49">
         <v>1</v>
       </c>
-      <c r="D20" s="47">
-        <v>0.86980000000000002</v>
-      </c>
-      <c r="E20" s="47">
-        <v>0.62109999999999999</v>
-      </c>
-      <c r="F20" s="47">
-        <v>0.62109999999999999</v>
-      </c>
-    </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B21" s="26" t="s">
-        <v>299</v>
-      </c>
-      <c r="C21" s="47">
+      <c r="E29" s="49">
+        <v>0.66815000000000002</v>
+      </c>
+      <c r="F29" s="49">
+        <v>0.42349999999999999</v>
+      </c>
+      <c r="G29" s="49">
+        <v>0.42349999999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B30" s="26" t="s">
+        <v>310</v>
+      </c>
+      <c r="C30" s="26" t="s">
+        <v>308</v>
+      </c>
+      <c r="D30" s="49">
         <v>1</v>
       </c>
-      <c r="D21" s="47">
-        <v>0.86980000000000002</v>
-      </c>
-      <c r="E21" s="47">
-        <v>0.74829999999999997</v>
-      </c>
-      <c r="F21" s="47">
-        <v>0.74829999999999997</v>
+      <c r="E30" s="49">
+        <v>0.97130000000000005</v>
+      </c>
+      <c r="F30" s="49">
+        <v>0.94384999999999997</v>
+      </c>
+      <c r="G30" s="49">
+        <v>0.94384999999999997</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B31" s="26" t="s">
+        <v>310</v>
+      </c>
+      <c r="C31" s="26" t="s">
+        <v>296</v>
+      </c>
+      <c r="D31" s="49">
+        <v>0.99995000000000001</v>
+      </c>
+      <c r="E31" s="49">
+        <v>0.6542</v>
+      </c>
+      <c r="F31" s="49">
+        <v>0.41410000000000002</v>
+      </c>
+      <c r="G31" s="49">
+        <v>0.41410000000000002</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B32" s="26" t="s">
+        <v>311</v>
+      </c>
+      <c r="C32" s="26" t="s">
+        <v>308</v>
+      </c>
+      <c r="D32" s="49">
+        <v>1</v>
+      </c>
+      <c r="E32" s="49">
+        <v>0.96435000000000004</v>
+      </c>
+      <c r="F32" s="49">
+        <v>0.93030000000000002</v>
+      </c>
+      <c r="G32" s="49">
+        <v>0.93030000000000002</v>
+      </c>
+    </row>
+    <row r="33" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B33" s="26" t="s">
+        <v>311</v>
+      </c>
+      <c r="C33" s="26" t="s">
+        <v>296</v>
+      </c>
+      <c r="D33" s="49">
+        <v>0.99990000000000001</v>
+      </c>
+      <c r="E33" s="49">
+        <v>0.61055000000000004</v>
+      </c>
+      <c r="F33" s="49">
+        <v>0.37695000000000001</v>
+      </c>
+      <c r="G33" s="49">
+        <v>0.37695000000000001</v>
+      </c>
+    </row>
+    <row r="34" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B34" s="26" t="s">
+        <v>312</v>
+      </c>
+      <c r="C34" s="26" t="s">
+        <v>308</v>
+      </c>
+      <c r="D34" s="49">
+        <v>0.99985000000000002</v>
+      </c>
+      <c r="E34" s="49">
+        <v>0.91244999999999998</v>
+      </c>
+      <c r="F34" s="49">
+        <v>0.86550000000000005</v>
+      </c>
+      <c r="G34" s="49">
+        <v>0.86550000000000005</v>
+      </c>
+    </row>
+    <row r="35" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B35" s="26" t="s">
+        <v>312</v>
+      </c>
+      <c r="C35" s="26" t="s">
+        <v>296</v>
+      </c>
+      <c r="D35" s="49">
+        <v>0.99570000000000003</v>
+      </c>
+      <c r="E35" s="49">
+        <v>0.50029999999999997</v>
+      </c>
+      <c r="F35" s="49">
+        <v>0.3024</v>
+      </c>
+      <c r="G35" s="49">
+        <v>0.3024</v>
+      </c>
+    </row>
+    <row r="38" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B38" s="25" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="39" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B39" s="50" t="s">
+        <v>308</v>
+      </c>
+      <c r="J39" s="50" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="40" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B40" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="J40" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="K40" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="L40" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="M40" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="N40" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="O40" s="4" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="41" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B41" s="31">
+        <v>0</v>
+      </c>
+      <c r="C41" s="32">
+        <v>144000</v>
+      </c>
+      <c r="D41" s="32">
+        <v>144000</v>
+      </c>
+      <c r="E41" s="32">
+        <v>144000</v>
+      </c>
+      <c r="F41" s="32">
+        <v>144000</v>
+      </c>
+      <c r="G41" s="32">
+        <v>144000</v>
+      </c>
+      <c r="J41" s="31">
+        <v>0</v>
+      </c>
+      <c r="K41" s="32">
+        <v>144000</v>
+      </c>
+      <c r="L41" s="32">
+        <v>144000</v>
+      </c>
+      <c r="M41" s="32">
+        <v>144000</v>
+      </c>
+      <c r="N41" s="32">
+        <v>144000</v>
+      </c>
+      <c r="O41" s="32">
+        <v>144000</v>
+      </c>
+    </row>
+    <row r="42" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B42" s="31">
+        <v>1</v>
+      </c>
+      <c r="C42" s="32">
+        <v>136454.11403771481</v>
+      </c>
+      <c r="D42" s="32">
+        <v>145546.7207558729</v>
+      </c>
+      <c r="E42" s="32">
+        <v>155716.37897509619</v>
+      </c>
+      <c r="F42" s="32">
+        <v>166313.6236591271</v>
+      </c>
+      <c r="G42" s="32">
+        <v>176050.47166730021</v>
+      </c>
+      <c r="J42" s="31">
+        <v>1</v>
+      </c>
+      <c r="K42" s="32">
+        <v>132358.11734650141</v>
+      </c>
+      <c r="L42" s="32">
+        <v>141172.33111916421</v>
+      </c>
+      <c r="M42" s="32">
+        <v>151010.86472015691</v>
+      </c>
+      <c r="N42" s="32">
+        <v>161267.09650384239</v>
+      </c>
+      <c r="O42" s="32">
+        <v>170682.91779692369</v>
+      </c>
+    </row>
+    <row r="43" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B43" s="31">
+        <v>2</v>
+      </c>
+      <c r="C43" s="32">
+        <v>149671.6070711785</v>
+      </c>
+      <c r="D43" s="32">
+        <v>162679.5136214451</v>
+      </c>
+      <c r="E43" s="32">
+        <v>178615.36062258441</v>
+      </c>
+      <c r="F43" s="32">
+        <v>195244.69905071979</v>
+      </c>
+      <c r="G43" s="32">
+        <v>211621.67220002229</v>
+      </c>
+      <c r="J43" s="31">
+        <v>2</v>
+      </c>
+      <c r="K43" s="32">
+        <v>141174.83687990959</v>
+      </c>
+      <c r="L43" s="32">
+        <v>153419.92590136011</v>
+      </c>
+      <c r="M43" s="32">
+        <v>168400.30970139091</v>
+      </c>
+      <c r="N43" s="32">
+        <v>184028.1179575948</v>
+      </c>
+      <c r="O43" s="32">
+        <v>199439.3961008481</v>
+      </c>
+    </row>
+    <row r="44" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B44" s="31">
+        <v>3</v>
+      </c>
+      <c r="C44" s="32">
+        <v>165345.95663557891</v>
+      </c>
+      <c r="D44" s="32">
+        <v>182118.44425340529</v>
+      </c>
+      <c r="E44" s="32">
+        <v>203316.66679781239</v>
+      </c>
+      <c r="F44" s="32">
+        <v>226051.60449960249</v>
+      </c>
+      <c r="G44" s="32">
+        <v>248357.98895150251</v>
+      </c>
+      <c r="J44" s="31">
+        <v>3</v>
+      </c>
+      <c r="K44" s="32">
+        <v>151892.07877474269</v>
+      </c>
+      <c r="L44" s="32">
+        <v>167218.0832245308</v>
+      </c>
+      <c r="M44" s="32">
+        <v>186587.892642363</v>
+      </c>
+      <c r="N44" s="32">
+        <v>207352.44143486471</v>
+      </c>
+      <c r="O44" s="32">
+        <v>227758.40235214701</v>
+      </c>
+    </row>
+    <row r="45" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B45" s="31">
+        <v>4</v>
+      </c>
+      <c r="C45" s="32">
+        <v>182419.22432318001</v>
+      </c>
+      <c r="D45" s="32">
+        <v>203529.11199860851</v>
+      </c>
+      <c r="E45" s="32">
+        <v>229941.20084669939</v>
+      </c>
+      <c r="F45" s="32">
+        <v>258860.78612988</v>
+      </c>
+      <c r="G45" s="32">
+        <v>288271.50712606887</v>
+      </c>
+      <c r="J45" s="31">
+        <v>4</v>
+      </c>
+      <c r="K45" s="32">
+        <v>163351.46814548699</v>
+      </c>
+      <c r="L45" s="32">
+        <v>182170.07745993219</v>
+      </c>
+      <c r="M45" s="32">
+        <v>205625.5463196979</v>
+      </c>
+      <c r="N45" s="32">
+        <v>231214.4907756061</v>
+      </c>
+      <c r="O45" s="32">
+        <v>257322.15900428299</v>
+      </c>
+    </row>
+    <row r="46" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B46" s="31">
+        <v>5</v>
+      </c>
+      <c r="C46" s="32">
+        <v>199689.55825826389</v>
+      </c>
+      <c r="D46" s="32">
+        <v>225812.48273427461</v>
+      </c>
+      <c r="E46" s="32">
+        <v>258541.40201989791</v>
+      </c>
+      <c r="F46" s="32">
+        <v>295487.02661359042</v>
+      </c>
+      <c r="G46" s="32">
+        <v>332315.73845461663</v>
+      </c>
+      <c r="J46" s="31">
+        <v>5</v>
+      </c>
+      <c r="K46" s="32">
+        <v>174596.68601252761</v>
+      </c>
+      <c r="L46" s="32">
+        <v>197110.7939690222</v>
+      </c>
+      <c r="M46" s="32">
+        <v>225379.44353605431</v>
+      </c>
+      <c r="N46" s="32">
+        <v>257295.26398709769</v>
+      </c>
+      <c r="O46" s="32">
+        <v>288881.52113130892</v>
+      </c>
+    </row>
+    <row r="47" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B47" s="31">
+        <v>6</v>
+      </c>
+      <c r="C47" s="32">
+        <v>219410.27809867371</v>
+      </c>
+      <c r="D47" s="32">
+        <v>249979.73296284981</v>
+      </c>
+      <c r="E47" s="32">
+        <v>289547.16838242719</v>
+      </c>
+      <c r="F47" s="32">
+        <v>333678.99006542529</v>
+      </c>
+      <c r="G47" s="32">
+        <v>379620.58061925019</v>
+      </c>
+      <c r="J47" s="31">
+        <v>6</v>
+      </c>
+      <c r="K47" s="32">
+        <v>187317.9810934354</v>
+      </c>
+      <c r="L47" s="32">
+        <v>212969.1966738379</v>
+      </c>
+      <c r="M47" s="32">
+        <v>246144.1572326938</v>
+      </c>
+      <c r="N47" s="32">
+        <v>283212.54000680638</v>
+      </c>
+      <c r="O47" s="32">
+        <v>321686.15938295232</v>
+      </c>
+    </row>
+    <row r="48" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B48" s="31">
+        <v>7</v>
+      </c>
+      <c r="C48" s="32">
+        <v>240419.17783803181</v>
+      </c>
+      <c r="D48" s="32">
+        <v>276066.65842505981</v>
+      </c>
+      <c r="E48" s="32">
+        <v>322860.29881220788</v>
+      </c>
+      <c r="F48" s="32">
+        <v>376379.5299027919</v>
+      </c>
+      <c r="G48" s="32">
+        <v>432771.81591624132</v>
+      </c>
+      <c r="J48" s="31">
+        <v>7</v>
+      </c>
+      <c r="K48" s="32">
+        <v>200472.08183031899</v>
+      </c>
+      <c r="L48" s="32">
+        <v>229624.78731478841</v>
+      </c>
+      <c r="M48" s="32">
+        <v>267949.33268909517</v>
+      </c>
+      <c r="N48" s="32">
+        <v>311586.41553581238</v>
+      </c>
+      <c r="O48" s="32">
+        <v>357578.15436422458</v>
+      </c>
+    </row>
+    <row r="49" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B49" s="31">
+        <v>8</v>
+      </c>
+      <c r="C49" s="32">
+        <v>262517.50543018628</v>
+      </c>
+      <c r="D49" s="32">
+        <v>304571.80758942798</v>
+      </c>
+      <c r="E49" s="32">
+        <v>358663.76011296897</v>
+      </c>
+      <c r="F49" s="32">
+        <v>422156.86900359462</v>
+      </c>
+      <c r="G49" s="32">
+        <v>489374.59258078638</v>
+      </c>
+      <c r="J49" s="31">
+        <v>8</v>
+      </c>
+      <c r="K49" s="32">
+        <v>213961.49467619229</v>
+      </c>
+      <c r="L49" s="32">
+        <v>247479.66775782729</v>
+      </c>
+      <c r="M49" s="32">
+        <v>290450.57669378573</v>
+      </c>
+      <c r="N49" s="32">
+        <v>340715.67473655072</v>
+      </c>
+      <c r="O49" s="32">
+        <v>394001.19883365522</v>
+      </c>
+    </row>
+    <row r="50" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B50" s="31">
+        <v>9</v>
+      </c>
+      <c r="C50" s="32">
+        <v>286193.05847900541</v>
+      </c>
+      <c r="D50" s="32">
+        <v>334213.43747500272</v>
+      </c>
+      <c r="E50" s="32">
+        <v>397298.57018818421</v>
+      </c>
+      <c r="F50" s="32">
+        <v>472304.13068839122</v>
+      </c>
+      <c r="G50" s="32">
+        <v>550908.48512842145</v>
+      </c>
+      <c r="J50" s="31">
+        <v>9</v>
+      </c>
+      <c r="K50" s="32">
+        <v>228074.1946171195</v>
+      </c>
+      <c r="L50" s="32">
+        <v>265266.92059872037</v>
+      </c>
+      <c r="M50" s="32">
+        <v>314147.86516454321</v>
+      </c>
+      <c r="N50" s="32">
+        <v>371944.86086429452</v>
+      </c>
+      <c r="O50" s="32">
+        <v>432463.62157045072</v>
+      </c>
+    </row>
+    <row r="51" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B51" s="31">
+        <v>10</v>
+      </c>
+      <c r="C51" s="32">
+        <v>311851.51402412099</v>
+      </c>
+      <c r="D51" s="32">
+        <v>366554.01477934461</v>
+      </c>
+      <c r="E51" s="32">
+        <v>438264.20737880259</v>
+      </c>
+      <c r="F51" s="32">
+        <v>524538.6908439768</v>
+      </c>
+      <c r="G51" s="32">
+        <v>618968.72940384422</v>
+      </c>
+      <c r="J51" s="31">
+        <v>10</v>
+      </c>
+      <c r="K51" s="32">
+        <v>242887.86952405519</v>
+      </c>
+      <c r="L51" s="32">
+        <v>284283.09972704097</v>
+      </c>
+      <c r="M51" s="32">
+        <v>338588.91969723091</v>
+      </c>
+      <c r="N51" s="32">
+        <v>403122.33047904988</v>
+      </c>
+      <c r="O51" s="32">
+        <v>474047.28289370378</v>
+      </c>
+    </row>
+    <row r="52" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B52" s="31">
+        <v>11</v>
+      </c>
+      <c r="C52" s="32">
+        <v>339943.60786837683</v>
+      </c>
+      <c r="D52" s="32">
+        <v>402625.15404770343</v>
+      </c>
+      <c r="E52" s="32">
+        <v>484754.69536159461</v>
+      </c>
+      <c r="F52" s="32">
+        <v>585106.20038470079</v>
+      </c>
+      <c r="G52" s="32">
+        <v>692461.61838036112</v>
+      </c>
+      <c r="J52" s="31">
+        <v>11</v>
+      </c>
+      <c r="K52" s="32">
+        <v>258920.9960379448</v>
+      </c>
+      <c r="L52" s="32">
+        <v>304948.50732605049</v>
+      </c>
+      <c r="M52" s="32">
+        <v>365376.00166761369</v>
+      </c>
+      <c r="N52" s="32">
+        <v>438260.8377906708</v>
+      </c>
+      <c r="O52" s="32">
+        <v>516979.29605962051</v>
+      </c>
+    </row>
+    <row r="53" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B53" s="31">
+        <v>12</v>
+      </c>
+      <c r="C53" s="32">
+        <v>369648.77492398949</v>
+      </c>
+      <c r="D53" s="32">
+        <v>438931.24224364187</v>
+      </c>
+      <c r="E53" s="32">
+        <v>533192.82607821259</v>
+      </c>
+      <c r="F53" s="32">
+        <v>649710.54003038676</v>
+      </c>
+      <c r="G53" s="32">
+        <v>773496.43855668011</v>
+      </c>
+      <c r="J53" s="31">
+        <v>12</v>
+      </c>
+      <c r="K53" s="32">
+        <v>275402.72575675469</v>
+      </c>
+      <c r="L53" s="32">
+        <v>325210.1353470562</v>
+      </c>
+      <c r="M53" s="32">
+        <v>392365.90427337523</v>
+      </c>
+      <c r="N53" s="32">
+        <v>475179.39732357248</v>
+      </c>
+      <c r="O53" s="32">
+        <v>563101.25735639769</v>
+      </c>
+    </row>
+    <row r="54" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B54" s="31">
+        <v>13</v>
+      </c>
+      <c r="C54" s="32">
+        <v>400537.70741422568</v>
+      </c>
+      <c r="D54" s="32">
+        <v>478220.44430127402</v>
+      </c>
+      <c r="E54" s="32">
+        <v>585834.16813507199</v>
+      </c>
+      <c r="F54" s="32">
+        <v>719138.05652550212</v>
+      </c>
+      <c r="G54" s="32">
+        <v>865265.749852504</v>
+      </c>
+      <c r="J54" s="31">
+        <v>13</v>
+      </c>
+      <c r="K54" s="32">
+        <v>291860.41856410698</v>
+      </c>
+      <c r="L54" s="32">
+        <v>345960.69734681858</v>
+      </c>
+      <c r="M54" s="32">
+        <v>420953.81567837932</v>
+      </c>
+      <c r="N54" s="32">
+        <v>513261.63564776478</v>
+      </c>
+      <c r="O54" s="32">
+        <v>613340.5496304431</v>
+      </c>
+    </row>
+    <row r="55" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B55" s="31">
+        <v>14</v>
+      </c>
+      <c r="C55" s="32">
+        <v>417357.09284013568</v>
+      </c>
+      <c r="D55" s="32">
+        <v>507507.01829387358</v>
+      </c>
+      <c r="E55" s="32">
+        <v>628629.10844905814</v>
+      </c>
+      <c r="F55" s="32">
+        <v>779861.00180054002</v>
+      </c>
+      <c r="G55" s="32">
+        <v>947364.58160986402</v>
+      </c>
+      <c r="J55" s="31">
+        <v>14</v>
+      </c>
+      <c r="K55" s="32">
+        <v>293358.0121816668</v>
+      </c>
+      <c r="L55" s="32">
+        <v>354559.94828780589</v>
+      </c>
+      <c r="M55" s="32">
+        <v>436784.49826389342</v>
+      </c>
+      <c r="N55" s="32">
+        <v>538696.09737915127</v>
+      </c>
+      <c r="O55" s="32">
+        <v>650937.48164195172</v>
+      </c>
+    </row>
+    <row r="56" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B56" s="31">
+        <v>15</v>
+      </c>
+      <c r="C56" s="32">
+        <v>440075.83785721491</v>
+      </c>
+      <c r="D56" s="32">
+        <v>537423.12280648481</v>
+      </c>
+      <c r="E56" s="32">
+        <v>673390.85694207833</v>
+      </c>
+      <c r="F56" s="32">
+        <v>848356.11811680789</v>
+      </c>
+      <c r="G56" s="32">
+        <v>1034374.71586807</v>
+      </c>
+      <c r="J56" s="31">
+        <v>15</v>
+      </c>
+      <c r="K56" s="32">
+        <v>297925.14779223042</v>
+      </c>
+      <c r="L56" s="32">
+        <v>362728.65324041707</v>
+      </c>
+      <c r="M56" s="32">
+        <v>452302.13517696387</v>
+      </c>
+      <c r="N56" s="32">
+        <v>566616.74088959605</v>
+      </c>
+      <c r="O56" s="32">
+        <v>688342.09575796139</v>
+      </c>
+    </row>
+    <row r="57" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B57" s="31">
+        <v>16</v>
+      </c>
+      <c r="C57" s="32">
+        <v>447387.13444896019</v>
+      </c>
+      <c r="D57" s="32">
+        <v>556516.73273564246</v>
+      </c>
+      <c r="E57" s="32">
+        <v>710012.83142528951</v>
+      </c>
+      <c r="F57" s="32">
+        <v>904485.11730330484</v>
+      </c>
+      <c r="G57" s="32">
+        <v>1121897.004993387</v>
+      </c>
+      <c r="J57" s="31">
+        <v>16</v>
+      </c>
+      <c r="K57" s="32">
+        <v>287621.1357098138</v>
+      </c>
+      <c r="L57" s="32">
+        <v>357861.08079072891</v>
+      </c>
+      <c r="M57" s="32">
+        <v>455899.60215377557</v>
+      </c>
+      <c r="N57" s="32">
+        <v>580188.66069645796</v>
+      </c>
+      <c r="O57" s="32">
+        <v>717726.13247474318</v>
+      </c>
+    </row>
+    <row r="58" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B58" s="31">
+        <v>17</v>
+      </c>
+      <c r="C58" s="32">
+        <v>455729.32246423292</v>
+      </c>
+      <c r="D58" s="32">
+        <v>577855.65971696889</v>
+      </c>
+      <c r="E58" s="32">
+        <v>748600.25892487506</v>
+      </c>
+      <c r="F58" s="32">
+        <v>963966.30936693563</v>
+      </c>
+      <c r="G58" s="32">
+        <v>1210182.5574922019</v>
+      </c>
+      <c r="J58" s="31">
+        <v>17</v>
+      </c>
+      <c r="K58" s="32">
+        <v>277177.07525715721</v>
+      </c>
+      <c r="L58" s="32">
+        <v>353125.69341902953</v>
+      </c>
+      <c r="M58" s="32">
+        <v>459486.07030779117</v>
+      </c>
+      <c r="N58" s="32">
+        <v>592745.223647448</v>
+      </c>
+      <c r="O58" s="32">
+        <v>743042.16329889779</v>
+      </c>
+    </row>
+    <row r="59" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B59" s="31">
+        <v>18</v>
+      </c>
+      <c r="C59" s="32">
+        <v>466747.70968791877</v>
+      </c>
+      <c r="D59" s="32">
+        <v>601157.52492004272</v>
+      </c>
+      <c r="E59" s="32">
+        <v>788298.33134348679</v>
+      </c>
+      <c r="F59" s="32">
+        <v>1033184.963518028</v>
+      </c>
+      <c r="G59" s="32">
+        <v>1304652.037527476</v>
+      </c>
+      <c r="J59" s="31">
+        <v>18</v>
+      </c>
+      <c r="K59" s="32">
+        <v>267592.76570170763</v>
+      </c>
+      <c r="L59" s="32">
+        <v>349022.64697775338</v>
+      </c>
+      <c r="M59" s="32">
+        <v>461018.15614970971</v>
+      </c>
+      <c r="N59" s="32">
+        <v>608368.28776776791</v>
+      </c>
+      <c r="O59" s="32">
+        <v>771535.79803266481</v>
+      </c>
+    </row>
+    <row r="60" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B60" s="31">
+        <v>19</v>
+      </c>
+      <c r="C60" s="32">
+        <v>492621.89893717878</v>
+      </c>
+      <c r="D60" s="32">
+        <v>641066.20677449508</v>
+      </c>
+      <c r="E60" s="32">
+        <v>846487.64486634079</v>
+      </c>
+      <c r="F60" s="32">
+        <v>1116586.951260546</v>
+      </c>
+      <c r="G60" s="32">
+        <v>1431851.241432854</v>
+      </c>
+      <c r="J60" s="31">
+        <v>19</v>
+      </c>
+      <c r="K60" s="32">
+        <v>272075.50438150932</v>
+      </c>
+      <c r="L60" s="32">
+        <v>358569.5991294689</v>
+      </c>
+      <c r="M60" s="32">
+        <v>478571.30220604548</v>
+      </c>
+      <c r="N60" s="32">
+        <v>635768.97557281819</v>
+      </c>
+      <c r="O60" s="32">
+        <v>818065.50037741906</v>
+      </c>
+    </row>
+    <row r="61" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B61" s="31">
+        <v>20</v>
+      </c>
+      <c r="C61" s="32">
+        <v>519460.42550449038</v>
+      </c>
+      <c r="D61" s="32">
+        <v>679894.0092888556</v>
+      </c>
+      <c r="E61" s="32">
+        <v>905902.13551780046</v>
+      </c>
+      <c r="F61" s="32">
+        <v>1211676.085084609</v>
+      </c>
+      <c r="G61" s="32">
+        <v>1568199.03330314</v>
+      </c>
+      <c r="J61" s="31">
+        <v>20</v>
+      </c>
+      <c r="K61" s="32">
+        <v>275866.75447558338</v>
+      </c>
+      <c r="L61" s="32">
+        <v>367062.42207747098</v>
+      </c>
+      <c r="M61" s="32">
+        <v>495019.12183202722</v>
+      </c>
+      <c r="N61" s="32">
+        <v>667227.17029190576</v>
+      </c>
+      <c r="O61" s="32">
+        <v>865316.80580397742</v>
+      </c>
+    </row>
+    <row r="62" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B62" s="31">
+        <v>21</v>
+      </c>
+      <c r="C62" s="32">
+        <v>552999.66420744348</v>
+      </c>
+      <c r="D62" s="32">
+        <v>726105.80878808815</v>
+      </c>
+      <c r="E62" s="32">
+        <v>976368.20617851254</v>
+      </c>
+      <c r="F62" s="32">
+        <v>1316154.300247669</v>
+      </c>
+      <c r="G62" s="32">
+        <v>1720575.6690432881</v>
+      </c>
+      <c r="J62" s="31">
+        <v>21</v>
+      </c>
+      <c r="K62" s="32">
+        <v>285161.73033259681</v>
+      </c>
+      <c r="L62" s="32">
+        <v>380072.41225775488</v>
+      </c>
+      <c r="M62" s="32">
+        <v>517521.68351575959</v>
+      </c>
+      <c r="N62" s="32">
+        <v>702355.15968918265</v>
+      </c>
+      <c r="O62" s="32">
+        <v>921863.7280852485</v>
+      </c>
+    </row>
+    <row r="63" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B63" s="31">
+        <v>22</v>
+      </c>
+      <c r="C63" s="32">
+        <v>587764.8493924503</v>
+      </c>
+      <c r="D63" s="32">
+        <v>778419.78169898526</v>
+      </c>
+      <c r="E63" s="32">
+        <v>1054109.793348694</v>
+      </c>
+      <c r="F63" s="32">
+        <v>1429263.130083642</v>
+      </c>
+      <c r="G63" s="32">
+        <v>1875782.796299756</v>
+      </c>
+      <c r="J63" s="31">
+        <v>22</v>
+      </c>
+      <c r="K63" s="32">
+        <v>294657.53604529361</v>
+      </c>
+      <c r="L63" s="32">
+        <v>394963.23749970627</v>
+      </c>
+      <c r="M63" s="32">
+        <v>541503.73070416716</v>
+      </c>
+      <c r="N63" s="32">
+        <v>739038.34266847465</v>
+      </c>
+      <c r="O63" s="32">
+        <v>975357.57286233362</v>
+      </c>
+    </row>
+    <row r="64" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B64" s="31">
+        <v>23</v>
+      </c>
+      <c r="C64" s="32">
+        <v>624176.92053188803</v>
+      </c>
+      <c r="D64" s="32">
+        <v>836745.75051655201</v>
+      </c>
+      <c r="E64" s="32">
+        <v>1136752.4824785979</v>
+      </c>
+      <c r="F64" s="32">
+        <v>1554786.9358183751</v>
+      </c>
+      <c r="G64" s="32">
+        <v>2046376.8137268189</v>
+      </c>
+      <c r="J64" s="31">
+        <v>23</v>
+      </c>
+      <c r="K64" s="32">
+        <v>303546.81170536962</v>
+      </c>
+      <c r="L64" s="32">
+        <v>412355.10737029533</v>
+      </c>
+      <c r="M64" s="32">
+        <v>565893.70431658032</v>
+      </c>
+      <c r="N64" s="32">
+        <v>779434.03524184844</v>
+      </c>
+      <c r="O64" s="32">
+        <v>1030060.964281491</v>
+      </c>
+    </row>
+    <row r="65" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B65" s="31">
+        <v>24</v>
+      </c>
+      <c r="C65" s="32">
+        <v>664167.46387587686</v>
+      </c>
+      <c r="D65" s="32">
+        <v>892044.77694465767</v>
+      </c>
+      <c r="E65" s="32">
+        <v>1224409.891552228</v>
+      </c>
+      <c r="F65" s="32">
+        <v>1679184.113114828</v>
+      </c>
+      <c r="G65" s="32">
+        <v>2225430.3316212692</v>
+      </c>
+      <c r="J65" s="31">
+        <v>24</v>
+      </c>
+      <c r="K65" s="32">
+        <v>313860.39851408137</v>
+      </c>
+      <c r="L65" s="32">
+        <v>426887.12660009589</v>
+      </c>
+      <c r="M65" s="32">
+        <v>591025.46134616877</v>
+      </c>
+      <c r="N65" s="32">
+        <v>815825.89433899405</v>
+      </c>
+      <c r="O65" s="32">
+        <v>1087650.948499074</v>
+      </c>
+    </row>
+    <row r="66" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B66" s="31">
+        <v>25</v>
+      </c>
+      <c r="C66" s="32">
+        <v>707660.27605145529</v>
+      </c>
+      <c r="D66" s="32">
+        <v>961391.90749138442</v>
+      </c>
+      <c r="E66" s="32">
+        <v>1320710.070178245</v>
+      </c>
+      <c r="F66" s="32">
+        <v>1827172.568253553</v>
+      </c>
+      <c r="G66" s="32">
+        <v>2423866.0635540918</v>
+      </c>
+      <c r="J66" s="31">
+        <v>25</v>
+      </c>
+      <c r="K66" s="32">
+        <v>324301.03100004949</v>
+      </c>
+      <c r="L66" s="32">
+        <v>445602.99573909678</v>
+      </c>
+      <c r="M66" s="32">
+        <v>617754.26608480699</v>
+      </c>
+      <c r="N66" s="32">
+        <v>861035.60000181326</v>
+      </c>
+      <c r="O66" s="32">
+        <v>1148464.697207463</v>
+      </c>
+    </row>
+    <row r="67" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B67" s="31">
+        <v>26</v>
+      </c>
+      <c r="C67" s="32">
+        <v>255670.9848559589</v>
+      </c>
+      <c r="D67" s="32">
+        <v>523590.39318202413</v>
+      </c>
+      <c r="E67" s="32">
+        <v>912158.1231031795</v>
+      </c>
+      <c r="F67" s="32">
+        <v>1468759.2576856001</v>
+      </c>
+      <c r="G67" s="32">
+        <v>2127025.4718987201</v>
+      </c>
+      <c r="J67" s="31">
+        <v>26</v>
+      </c>
+      <c r="K67" s="32">
+        <v>0</v>
+      </c>
+      <c r="L67" s="32">
+        <v>0</v>
+      </c>
+      <c r="M67" s="32">
+        <v>153286.36311925211</v>
+      </c>
+      <c r="N67" s="32">
+        <v>409623.99551416212</v>
+      </c>
+      <c r="O67" s="32">
+        <v>717887.46810933622</v>
+      </c>
+    </row>
+    <row r="68" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B68" s="31">
+        <v>27</v>
+      </c>
+      <c r="C68" s="32">
+        <v>272440.71148612868</v>
+      </c>
+      <c r="D68" s="32">
+        <v>559107.56156578904</v>
+      </c>
+      <c r="E68" s="32">
+        <v>982174.09242948447</v>
+      </c>
+      <c r="F68" s="32">
+        <v>1587614.464996669</v>
+      </c>
+      <c r="G68" s="32">
+        <v>2314336.427245236</v>
+      </c>
+      <c r="J68" s="31">
+        <v>27</v>
+      </c>
+      <c r="K68" s="32">
+        <v>0</v>
+      </c>
+      <c r="L68" s="32">
+        <v>0</v>
+      </c>
+      <c r="M68" s="32">
+        <v>159008.57522110999</v>
+      </c>
+      <c r="N68" s="32">
+        <v>426188.93914576247</v>
+      </c>
+      <c r="O68" s="32">
+        <v>748570.2207656909</v>
+      </c>
+    </row>
+    <row r="69" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B69" s="31">
+        <v>28</v>
+      </c>
+      <c r="C69" s="32">
+        <v>290273.06024275877</v>
+      </c>
+      <c r="D69" s="32">
+        <v>596553.32054687815</v>
+      </c>
+      <c r="E69" s="32">
+        <v>1055483.069819591</v>
+      </c>
+      <c r="F69" s="32">
+        <v>1718131.2284537631</v>
+      </c>
+      <c r="G69" s="32">
+        <v>2508219.0119728828</v>
+      </c>
+      <c r="J69" s="31">
+        <v>28</v>
+      </c>
+      <c r="K69" s="32">
+        <v>0</v>
+      </c>
+      <c r="L69" s="32">
+        <v>0</v>
+      </c>
+      <c r="M69" s="32">
+        <v>164396.56207811521</v>
+      </c>
+      <c r="N69" s="32">
+        <v>445146.0160144855</v>
+      </c>
+      <c r="O69" s="32">
+        <v>786425.2092011557</v>
+      </c>
+    </row>
+    <row r="70" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B70" s="31">
+        <v>29</v>
+      </c>
+      <c r="C70" s="32">
+        <v>308912.11747827928</v>
+      </c>
+      <c r="D70" s="32">
+        <v>640756.88628192258</v>
+      </c>
+      <c r="E70" s="32">
+        <v>1140301.48207127</v>
+      </c>
+      <c r="F70" s="32">
+        <v>1855872.6222613929</v>
+      </c>
+      <c r="G70" s="32">
+        <v>2761555.3662512079</v>
+      </c>
+      <c r="J70" s="31">
+        <v>29</v>
+      </c>
+      <c r="K70" s="32">
+        <v>0</v>
+      </c>
+      <c r="L70" s="32">
+        <v>0</v>
+      </c>
+      <c r="M70" s="32">
+        <v>172313.46196586659</v>
+      </c>
+      <c r="N70" s="32">
+        <v>464654.92239961942</v>
+      </c>
+      <c r="O70" s="32">
+        <v>829601.46116567799</v>
+      </c>
+    </row>
+    <row r="71" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B71" s="31">
+        <v>30</v>
+      </c>
+      <c r="C71" s="32">
+        <v>333212.99037842039</v>
+      </c>
+      <c r="D71" s="32">
+        <v>688703.15408531029</v>
+      </c>
+      <c r="E71" s="32">
+        <v>1224331.7453612019</v>
+      </c>
+      <c r="F71" s="32">
+        <v>2019278.4222586099</v>
+      </c>
+      <c r="G71" s="32">
+        <v>2999698.42570135</v>
+      </c>
+      <c r="J71" s="31">
+        <v>30</v>
+      </c>
+      <c r="K71" s="32">
+        <v>0</v>
+      </c>
+      <c r="L71" s="32">
+        <v>0</v>
+      </c>
+      <c r="M71" s="32">
+        <v>180058.15022790921</v>
+      </c>
+      <c r="N71" s="32">
+        <v>490053.71824872901</v>
+      </c>
+      <c r="O71" s="32">
+        <v>879270.4017871744</v>
+      </c>
+    </row>
+    <row r="72" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B72" s="31">
+        <v>31</v>
+      </c>
+      <c r="C72" s="32">
+        <v>355265.84577457153</v>
+      </c>
+      <c r="D72" s="32">
+        <v>737503.29627111612</v>
+      </c>
+      <c r="E72" s="32">
+        <v>1317746.031404275</v>
+      </c>
+      <c r="F72" s="32">
+        <v>2181855.9318649122</v>
+      </c>
+      <c r="G72" s="32">
+        <v>3256825.1084248442</v>
+      </c>
+      <c r="J72" s="31">
+        <v>31</v>
+      </c>
+      <c r="K72" s="32">
+        <v>0</v>
+      </c>
+      <c r="L72" s="32">
+        <v>0</v>
+      </c>
+      <c r="M72" s="32">
+        <v>188158.26131765131</v>
+      </c>
+      <c r="N72" s="32">
+        <v>515119.71328417922</v>
+      </c>
+      <c r="O72" s="32">
+        <v>924330.98658551031</v>
+      </c>
+    </row>
+    <row r="73" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B73" s="31">
+        <v>32</v>
+      </c>
+      <c r="C73" s="32">
+        <v>380689.82776569371</v>
+      </c>
+      <c r="D73" s="32">
+        <v>788157.30568670877</v>
+      </c>
+      <c r="E73" s="32">
+        <v>1422930.0503417561</v>
+      </c>
+      <c r="F73" s="32">
+        <v>2360410.53529432</v>
+      </c>
+      <c r="G73" s="32">
+        <v>3553467.573872644</v>
+      </c>
+      <c r="J73" s="31">
+        <v>32</v>
+      </c>
+      <c r="K73" s="32">
+        <v>0</v>
+      </c>
+      <c r="L73" s="32">
+        <v>0</v>
+      </c>
+      <c r="M73" s="32">
+        <v>196588.1718983255</v>
+      </c>
+      <c r="N73" s="32">
+        <v>536321.58364519454</v>
+      </c>
+      <c r="O73" s="32">
+        <v>975456.03702214942</v>
+      </c>
+    </row>
+    <row r="74" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B74" s="31">
+        <v>33</v>
+      </c>
+      <c r="C74" s="32">
+        <v>408799.13188907033</v>
+      </c>
+      <c r="D74" s="32">
+        <v>845468.36011497187</v>
+      </c>
+      <c r="E74" s="32">
+        <v>1531764.363825772</v>
+      </c>
+      <c r="F74" s="32">
+        <v>2547919.366632849</v>
+      </c>
+      <c r="G74" s="32">
+        <v>3867853.3682618332</v>
+      </c>
+      <c r="J74" s="31">
+        <v>33</v>
+      </c>
+      <c r="K74" s="32">
+        <v>0</v>
+      </c>
+      <c r="L74" s="32">
+        <v>0</v>
+      </c>
+      <c r="M74" s="32">
+        <v>204152.69952207521</v>
+      </c>
+      <c r="N74" s="32">
+        <v>561023.96546600712</v>
+      </c>
+      <c r="O74" s="32">
+        <v>1014123.056282845</v>
+      </c>
+    </row>
+    <row r="75" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B75" s="31">
+        <v>34</v>
+      </c>
+      <c r="C75" s="32">
+        <v>438692.44752603368</v>
+      </c>
+      <c r="D75" s="32">
+        <v>904156.56138106412</v>
+      </c>
+      <c r="E75" s="32">
+        <v>1649056.212047155</v>
+      </c>
+      <c r="F75" s="32">
+        <v>2759067.789268943</v>
+      </c>
+      <c r="G75" s="32">
+        <v>4223370.9169281572</v>
+      </c>
+      <c r="J75" s="31">
+        <v>34</v>
+      </c>
+      <c r="K75" s="32">
+        <v>0</v>
+      </c>
+      <c r="L75" s="32">
+        <v>0</v>
+      </c>
+      <c r="M75" s="32">
+        <v>212807.4237549869</v>
+      </c>
+      <c r="N75" s="32">
+        <v>586784.55288527138</v>
+      </c>
+      <c r="O75" s="32">
+        <v>1070527.870974534</v>
+      </c>
+    </row>
+    <row r="76" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B76" s="31">
+        <v>35</v>
+      </c>
+      <c r="C76" s="32">
+        <v>466480.00734621898</v>
+      </c>
+      <c r="D76" s="32">
+        <v>973176.91438967898</v>
+      </c>
+      <c r="E76" s="32">
+        <v>1773413.1529597591</v>
+      </c>
+      <c r="F76" s="32">
+        <v>2993111.0398661499</v>
+      </c>
+      <c r="G76" s="32">
+        <v>4586987.72590914</v>
+      </c>
+      <c r="J76" s="31">
+        <v>35</v>
+      </c>
+      <c r="K76" s="32">
+        <v>0</v>
+      </c>
+      <c r="L76" s="32">
+        <v>0</v>
+      </c>
+      <c r="M76" s="32">
+        <v>220605.15994680021</v>
+      </c>
+      <c r="N76" s="32">
+        <v>613206.06709132367</v>
+      </c>
+      <c r="O76" s="32">
+        <v>1126573.534523322</v>
+      </c>
+    </row>
+    <row r="77" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B77" s="31">
+        <v>36</v>
+      </c>
+      <c r="C77" s="32">
+        <v>503474.08793131309</v>
+      </c>
+      <c r="D77" s="32">
+        <v>1041387.833513363</v>
+      </c>
+      <c r="E77" s="32">
+        <v>1918066.122944931</v>
+      </c>
+      <c r="F77" s="32">
+        <v>3238512.6598543422</v>
+      </c>
+      <c r="G77" s="32">
+        <v>5013503.6097666528</v>
+      </c>
+      <c r="J77" s="31">
+        <v>36</v>
+      </c>
+      <c r="K77" s="32">
+        <v>0</v>
+      </c>
+      <c r="L77" s="32">
+        <v>0</v>
+      </c>
+      <c r="M77" s="32">
+        <v>230251.9088631201</v>
+      </c>
+      <c r="N77" s="32">
+        <v>645558.55278608622</v>
+      </c>
+      <c r="O77" s="32">
+        <v>1190450.159143731</v>
+      </c>
+    </row>
+    <row r="78" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B78" s="31">
+        <v>37</v>
+      </c>
+      <c r="C78" s="32">
+        <v>536307.27569414803</v>
+      </c>
+      <c r="D78" s="32">
+        <v>1117828.7393510169</v>
+      </c>
+      <c r="E78" s="32">
+        <v>2066446.827250693</v>
+      </c>
+      <c r="F78" s="32">
+        <v>3515074.8124660398</v>
+      </c>
+      <c r="G78" s="32">
+        <v>5445545.7016117312</v>
+      </c>
+      <c r="J78" s="31">
+        <v>37</v>
+      </c>
+      <c r="K78" s="32">
+        <v>0</v>
+      </c>
+      <c r="L78" s="32">
+        <v>0</v>
+      </c>
+      <c r="M78" s="32">
+        <v>239603.4355525717</v>
+      </c>
+      <c r="N78" s="32">
+        <v>676561.66535542463</v>
+      </c>
+      <c r="O78" s="32">
+        <v>1255466.357932514</v>
+      </c>
+    </row>
+    <row r="79" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B79" s="31">
+        <v>38</v>
+      </c>
+      <c r="C79" s="32">
+        <v>569410.7845699141</v>
+      </c>
+      <c r="D79" s="32">
+        <v>1191501.5827798061</v>
+      </c>
+      <c r="E79" s="32">
+        <v>2220185.697328453</v>
+      </c>
+      <c r="F79" s="32">
+        <v>3797859.504405804</v>
+      </c>
+      <c r="G79" s="32">
+        <v>5875463.2557453858</v>
+      </c>
+      <c r="J79" s="31">
+        <v>38</v>
+      </c>
+      <c r="K79" s="32">
+        <v>0</v>
+      </c>
+      <c r="L79" s="32">
+        <v>0</v>
+      </c>
+      <c r="M79" s="32">
+        <v>251367.8437608126</v>
+      </c>
+      <c r="N79" s="32">
+        <v>707700.05449081771</v>
+      </c>
+      <c r="O79" s="32">
+        <v>1321750.638917235</v>
+      </c>
+    </row>
+    <row r="80" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B80" s="31">
+        <v>39</v>
+      </c>
+      <c r="C80" s="32">
+        <v>615584.30652590259</v>
+      </c>
+      <c r="D80" s="32">
+        <v>1290069.9632471369</v>
+      </c>
+      <c r="E80" s="32">
+        <v>2382688.564175752</v>
+      </c>
+      <c r="F80" s="32">
+        <v>4104778.516752</v>
+      </c>
+      <c r="G80" s="32">
+        <v>6470027.6809031526</v>
+      </c>
+      <c r="J80" s="31">
+        <v>39</v>
+      </c>
+      <c r="K80" s="32">
+        <v>0</v>
+      </c>
+      <c r="L80" s="32">
+        <v>0</v>
+      </c>
+      <c r="M80" s="32">
+        <v>262542.16323634249</v>
+      </c>
+      <c r="N80" s="32">
+        <v>741781.95713108929</v>
+      </c>
+      <c r="O80" s="32">
+        <v>1386251.649922325</v>
+      </c>
+    </row>
+    <row r="81" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B81" s="31">
+        <v>40</v>
+      </c>
+      <c r="C81" s="32">
+        <v>654732.70775104361</v>
+      </c>
+      <c r="D81" s="32">
+        <v>1387152.4019598169</v>
+      </c>
+      <c r="E81" s="32">
+        <v>2580933.266235474</v>
+      </c>
+      <c r="F81" s="32">
+        <v>4431469.4183793738</v>
+      </c>
+      <c r="G81" s="32">
+        <v>6992865.8326747734</v>
+      </c>
+      <c r="J81" s="31">
+        <v>40</v>
+      </c>
+      <c r="K81" s="32">
+        <v>0</v>
+      </c>
+      <c r="L81" s="32">
+        <v>0</v>
+      </c>
+      <c r="M81" s="32">
+        <v>274534.0743478951</v>
+      </c>
+      <c r="N81" s="32">
+        <v>771874.81542561506</v>
+      </c>
+      <c r="O81" s="32">
+        <v>1464076.351041272</v>
+      </c>
+    </row>
+    <row r="82" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B82" s="31">
+        <v>41</v>
+      </c>
+      <c r="C82" s="32">
+        <v>702719.43423285394</v>
+      </c>
+      <c r="D82" s="32">
+        <v>1484050.2368170971</v>
+      </c>
+      <c r="E82" s="32">
+        <v>2777344.327436646</v>
+      </c>
+      <c r="F82" s="32">
+        <v>4824483.7287606923</v>
+      </c>
+      <c r="G82" s="32">
+        <v>7616960.196385242</v>
+      </c>
+      <c r="J82" s="31">
+        <v>41</v>
+      </c>
+      <c r="K82" s="32">
+        <v>0</v>
+      </c>
+      <c r="L82" s="32">
+        <v>0</v>
+      </c>
+      <c r="M82" s="32">
+        <v>286998.31748267898</v>
+      </c>
+      <c r="N82" s="32">
+        <v>809714.25876119966</v>
+      </c>
+      <c r="O82" s="32">
+        <v>1528996.0021223619</v>
+      </c>
+    </row>
+    <row r="83" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B83" s="31">
+        <v>42</v>
+      </c>
+      <c r="C83" s="32">
+        <v>750163.32987731055</v>
+      </c>
+      <c r="D83" s="32">
+        <v>1593743.3205952609</v>
+      </c>
+      <c r="E83" s="32">
+        <v>2993700.371465933</v>
+      </c>
+      <c r="F83" s="32">
+        <v>5195361.0528021324</v>
+      </c>
+      <c r="G83" s="32">
+        <v>8259579.594608455</v>
+      </c>
+      <c r="J83" s="31">
+        <v>42</v>
+      </c>
+      <c r="K83" s="32">
+        <v>0</v>
+      </c>
+      <c r="L83" s="32">
+        <v>0</v>
+      </c>
+      <c r="M83" s="32">
+        <v>298546.33544770879</v>
+      </c>
+      <c r="N83" s="32">
+        <v>843744.98733295535</v>
+      </c>
+      <c r="O83" s="32">
+        <v>1611760.22036105</v>
+      </c>
+    </row>
+    <row r="84" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B84" s="31">
+        <v>43</v>
+      </c>
+      <c r="C84" s="32">
+        <v>801827.0200714363</v>
+      </c>
+      <c r="D84" s="32">
+        <v>1712654.3048756339</v>
+      </c>
+      <c r="E84" s="32">
+        <v>3221770.7219450241</v>
+      </c>
+      <c r="F84" s="32">
+        <v>5621321.0707345624</v>
+      </c>
+      <c r="G84" s="32">
+        <v>8983064.201986175</v>
+      </c>
+      <c r="J84" s="31">
+        <v>43</v>
+      </c>
+      <c r="K84" s="32">
+        <v>0</v>
+      </c>
+      <c r="L84" s="32">
+        <v>0</v>
+      </c>
+      <c r="M84" s="32">
+        <v>312879.48939570918</v>
+      </c>
+      <c r="N84" s="32">
+        <v>881224.30409636372</v>
+      </c>
+      <c r="O84" s="32">
+        <v>1695180.6563732331</v>
+      </c>
+    </row>
+    <row r="85" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B85" s="31">
+        <v>44</v>
+      </c>
+      <c r="C85" s="32">
+        <v>857074.69807235978</v>
+      </c>
+      <c r="D85" s="32">
+        <v>1835896.4193475549</v>
+      </c>
+      <c r="E85" s="32">
+        <v>3477877.0126096471</v>
+      </c>
+      <c r="F85" s="32">
+        <v>6084626.4418700188</v>
+      </c>
+      <c r="G85" s="32">
+        <v>9758452.6571366359</v>
+      </c>
+      <c r="J85" s="31">
+        <v>44</v>
+      </c>
+      <c r="K85" s="32">
+        <v>0</v>
+      </c>
+      <c r="L85" s="32">
+        <v>0</v>
+      </c>
+      <c r="M85" s="32">
+        <v>326256.46374454192</v>
+      </c>
+      <c r="N85" s="32">
+        <v>920197.51945008663</v>
+      </c>
+      <c r="O85" s="32">
+        <v>1785805.186109843</v>
+      </c>
+    </row>
+    <row r="86" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B86" s="31">
+        <v>45</v>
+      </c>
+      <c r="C86" s="32">
+        <v>915506.22765419655</v>
+      </c>
+      <c r="D86" s="32">
+        <v>1964099.960523444</v>
+      </c>
+      <c r="E86" s="32">
+        <v>3731155.8650167701</v>
+      </c>
+      <c r="F86" s="32">
+        <v>6580027.4839586262</v>
+      </c>
+      <c r="G86" s="32">
+        <v>10649229.568028759</v>
+      </c>
+      <c r="J86" s="31">
+        <v>45</v>
+      </c>
+      <c r="K86" s="32">
+        <v>0</v>
+      </c>
+      <c r="L86" s="32">
+        <v>0</v>
+      </c>
+      <c r="M86" s="32">
+        <v>340253.55145231402</v>
+      </c>
+      <c r="N86" s="32">
+        <v>966062.14202981803</v>
+      </c>
+      <c r="O86" s="32">
+        <v>1871955.388266407</v>
+      </c>
+    </row>
+    <row r="87" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B87" s="31">
+        <v>46</v>
+      </c>
+      <c r="C87" s="32">
+        <v>984762.36517690285</v>
+      </c>
+      <c r="D87" s="32">
+        <v>2109113.0729337018</v>
+      </c>
+      <c r="E87" s="32">
+        <v>4024098.8446913208</v>
+      </c>
+      <c r="F87" s="32">
+        <v>7117968.9589581406</v>
+      </c>
+      <c r="G87" s="32">
+        <v>11515278.713286379</v>
+      </c>
+      <c r="J87" s="31">
+        <v>46</v>
+      </c>
+      <c r="K87" s="32">
+        <v>0</v>
+      </c>
+      <c r="L87" s="32">
+        <v>0</v>
+      </c>
+      <c r="M87" s="32">
+        <v>352449.61627208733</v>
+      </c>
+      <c r="N87" s="32">
+        <v>1009475.392205246</v>
+      </c>
+      <c r="O87" s="32">
+        <v>1973142.417860637</v>
+      </c>
+    </row>
+    <row r="88" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B88" s="31">
+        <v>47</v>
+      </c>
+      <c r="C88" s="32">
+        <v>1058211.4450268231</v>
+      </c>
+      <c r="D88" s="32">
+        <v>2268077.9298965121</v>
+      </c>
+      <c r="E88" s="32">
+        <v>4333332.1656370303</v>
+      </c>
+      <c r="F88" s="32">
+        <v>7710417.7802118165</v>
+      </c>
+      <c r="G88" s="32">
+        <v>12474746.696518149</v>
+      </c>
+      <c r="J88" s="31">
+        <v>47</v>
+      </c>
+      <c r="K88" s="32">
+        <v>0</v>
+      </c>
+      <c r="L88" s="32">
+        <v>0</v>
+      </c>
+      <c r="M88" s="32">
+        <v>367726.23773550871</v>
+      </c>
+      <c r="N88" s="32">
+        <v>1062539.1155425189</v>
+      </c>
+      <c r="O88" s="32">
+        <v>2067611.3885422519</v>
+      </c>
+    </row>
+    <row r="89" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B89" s="31">
+        <v>48</v>
+      </c>
+      <c r="C89" s="32">
+        <v>1141060.436490231</v>
+      </c>
+      <c r="D89" s="32">
+        <v>2439413.899661635</v>
+      </c>
+      <c r="E89" s="32">
+        <v>4675868.0944193052</v>
+      </c>
+      <c r="F89" s="32">
+        <v>8344285.5388264637</v>
+      </c>
+      <c r="G89" s="32">
+        <v>13522403.05906168</v>
+      </c>
+      <c r="J89" s="31">
+        <v>48</v>
+      </c>
+      <c r="K89" s="32">
+        <v>0</v>
+      </c>
+      <c r="L89" s="32">
+        <v>0</v>
+      </c>
+      <c r="M89" s="32">
+        <v>382112.91557670262</v>
+      </c>
+      <c r="N89" s="32">
+        <v>1111874.7224475159</v>
+      </c>
+      <c r="O89" s="32">
+        <v>2167146.9422424519</v>
+      </c>
+    </row>
+    <row r="90" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B90" s="31">
+        <v>49</v>
+      </c>
+      <c r="C90" s="32">
+        <v>1218444.402740445</v>
+      </c>
+      <c r="D90" s="32">
+        <v>2622355.7499031508</v>
+      </c>
+      <c r="E90" s="32">
+        <v>5035875.6388349701</v>
+      </c>
+      <c r="F90" s="32">
+        <v>8954018.4334737211</v>
+      </c>
+      <c r="G90" s="32">
+        <v>14639432.610328101</v>
+      </c>
+      <c r="J90" s="31">
+        <v>49</v>
+      </c>
+      <c r="K90" s="32">
+        <v>0</v>
+      </c>
+      <c r="L90" s="32">
+        <v>0</v>
+      </c>
+      <c r="M90" s="32">
+        <v>400072.030485756</v>
+      </c>
+      <c r="N90" s="32">
+        <v>1158486.4139444991</v>
+      </c>
+      <c r="O90" s="32">
+        <v>2275507.0447248351</v>
+      </c>
+    </row>
+    <row r="91" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B91" s="31">
+        <v>50</v>
+      </c>
+      <c r="C91" s="32">
+        <v>1311231.8202823671</v>
+      </c>
+      <c r="D91" s="32">
+        <v>2802980.66423178</v>
+      </c>
+      <c r="E91" s="32">
+        <v>5448079.025805857</v>
+      </c>
+      <c r="F91" s="32">
+        <v>9698456.4492181595</v>
+      </c>
+      <c r="G91" s="32">
+        <v>15889098.76650925</v>
+      </c>
+      <c r="J91" s="31">
+        <v>50</v>
+      </c>
+      <c r="K91" s="32">
+        <v>0</v>
+      </c>
+      <c r="L91" s="32">
+        <v>0</v>
+      </c>
+      <c r="M91" s="32">
+        <v>414317.88061139139</v>
+      </c>
+      <c r="N91" s="32">
+        <v>1208594.897917751</v>
+      </c>
+      <c r="O91" s="32">
+        <v>2387510.6395634999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
TIR requerida sobre el capital invertido (USD 144.000)
Acordado con el profesor guía: la reserva de 4% no financia metas, así que la TIR y la
factibilidad usan el mismo capital que el Montecarlo. TIR base 4,56% -> 4,65%; escenario
exigente 5,6% -> 5,7%; cobertura 0,61x -> 0,60x. objetivos.py, fórmula del Excel (02_Objetivos_TIR),
tir_capital_invertido.py (actualiza solo las tablas de objetivos), informe e insumos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T5hAYzxrHpdpyuLVyANGG6
</commit_message>
<xml_diff>
--- a/nexum_proyecto_final/modelo/Modelo_Nexum_v2.xlsx
+++ b/nexum_proyecto_final/modelo/Modelo_Nexum_v2.xlsx
@@ -592,7 +592,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Grupo 11 · ESF 2026-2 · Datos al 31-ago-2026 · Generado 09-10-2026 con codigo/run_all.py + excel_modelo.py</t>
+          <t>Grupo 11 · ESF 2026-2 · Datos al 31-ago-2026 · Generado 11-10-2026 con codigo/run_all.py + excel_modelo.py</t>
         </is>
       </c>
     </row>
@@ -3385,7 +3385,7 @@
         </is>
       </c>
       <c r="N7" s="27" t="n">
-        <v>0.045564080984627</v>
+        <v>0.04653130500365561</v>
       </c>
     </row>
     <row r="8">
@@ -3404,7 +3404,7 @@
         </is>
       </c>
       <c r="N8" s="27" t="n">
-        <v>0.04930438691645928</v>
+        <v>0.05034109182863089</v>
       </c>
     </row>
     <row r="9">
@@ -3423,7 +3423,7 @@
         </is>
       </c>
       <c r="N9" s="27" t="n">
-        <v>0.04934401368977564</v>
+        <v>0.05040198647251756</v>
       </c>
     </row>
     <row r="10">
@@ -3433,7 +3433,7 @@
         </is>
       </c>
       <c r="N10" s="27" t="n">
-        <v>0.04980583351961895</v>
+        <v>0.05085108572178737</v>
       </c>
     </row>
     <row r="11">
@@ -3443,7 +3443,7 @@
         </is>
       </c>
       <c r="N11" s="27" t="n">
-        <v>0.05369146964416108</v>
+        <v>0.0548303552432743</v>
       </c>
     </row>
     <row r="12">
@@ -3503,7 +3503,7 @@
         </is>
       </c>
       <c r="N12" s="27" t="n">
-        <v>0.05622355851730596</v>
+        <v>0.05740907235642809</v>
       </c>
     </row>
     <row r="13">
@@ -3511,7 +3511,7 @@
         <v>0</v>
       </c>
       <c r="C13" s="21">
-        <f>IF(B13=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B13=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D13" s="21">
@@ -3552,7 +3552,7 @@
         </is>
       </c>
       <c r="N13" s="27" t="n">
-        <v>0.04061423840906504</v>
+        <v>0.04165024480575189</v>
       </c>
     </row>
     <row r="14">
@@ -3560,7 +3560,7 @@
         <v>1</v>
       </c>
       <c r="C14" s="21">
-        <f>IF(B14=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B14=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D14" s="21">
@@ -3601,7 +3601,7 @@
         </is>
       </c>
       <c r="N14" s="27" t="n">
-        <v>0.03921642310646538</v>
+        <v>0.04010861685587032</v>
       </c>
     </row>
     <row r="15">
@@ -3609,7 +3609,7 @@
         <v>2</v>
       </c>
       <c r="C15" s="21">
-        <f>IF(B15=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B15=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D15" s="21">
@@ -3650,7 +3650,7 @@
         </is>
       </c>
       <c r="N15" s="27" t="n">
-        <v>0.03279627602421104</v>
+        <v>0.03375724729087864</v>
       </c>
     </row>
     <row r="16">
@@ -3658,7 +3658,7 @@
         <v>3</v>
       </c>
       <c r="C16" s="21">
-        <f>IF(B16=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B16=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D16" s="21">
@@ -3699,7 +3699,7 @@
         <v>4</v>
       </c>
       <c r="C17" s="21">
-        <f>IF(B17=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B17=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D17" s="21">
@@ -3740,7 +3740,7 @@
         <v>5</v>
       </c>
       <c r="C18" s="21">
-        <f>IF(B18=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B18=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D18" s="21">
@@ -3786,7 +3786,7 @@
         <v>6</v>
       </c>
       <c r="C19" s="21">
-        <f>IF(B19=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B19=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D19" s="21">
@@ -3852,7 +3852,7 @@
         <v>7</v>
       </c>
       <c r="C20" s="21">
-        <f>IF(B20=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B20=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D20" s="21">
@@ -3910,7 +3910,7 @@
         <v>8</v>
       </c>
       <c r="C21" s="21">
-        <f>IF(B21=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B21=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D21" s="21">
@@ -3968,7 +3968,7 @@
         <v>9</v>
       </c>
       <c r="C22" s="21">
-        <f>IF(B22=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B22=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D22" s="21">
@@ -4026,7 +4026,7 @@
         <v>10</v>
       </c>
       <c r="C23" s="21">
-        <f>IF(B23=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B23=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D23" s="21">
@@ -4084,7 +4084,7 @@
         <v>11</v>
       </c>
       <c r="C24" s="21">
-        <f>IF(B24=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B24=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D24" s="21">
@@ -4142,7 +4142,7 @@
         <v>12</v>
       </c>
       <c r="C25" s="21">
-        <f>IF(B25=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B25=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D25" s="21">
@@ -4200,7 +4200,7 @@
         <v>13</v>
       </c>
       <c r="C26" s="21">
-        <f>IF(B26=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B26=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D26" s="21">
@@ -4258,7 +4258,7 @@
         <v>14</v>
       </c>
       <c r="C27" s="21">
-        <f>IF(B27=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B27=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D27" s="21">
@@ -4316,7 +4316,7 @@
         <v>15</v>
       </c>
       <c r="C28" s="21">
-        <f>IF(B28=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B28=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D28" s="21">
@@ -4374,7 +4374,7 @@
         <v>16</v>
       </c>
       <c r="C29" s="21">
-        <f>IF(B29=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B29=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D29" s="21">
@@ -4415,7 +4415,7 @@
         <v>17</v>
       </c>
       <c r="C30" s="21">
-        <f>IF(B30=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B30=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D30" s="21">
@@ -4456,7 +4456,7 @@
         <v>18</v>
       </c>
       <c r="C31" s="21">
-        <f>IF(B31=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B31=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D31" s="21">
@@ -4497,7 +4497,7 @@
         <v>19</v>
       </c>
       <c r="C32" s="21">
-        <f>IF(B32=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B32=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D32" s="21">
@@ -4538,7 +4538,7 @@
         <v>20</v>
       </c>
       <c r="C33" s="21">
-        <f>IF(B33=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B33=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D33" s="21">
@@ -4584,7 +4584,7 @@
         <v>21</v>
       </c>
       <c r="C34" s="21">
-        <f>IF(B34=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B34=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D34" s="21">
@@ -4625,7 +4625,7 @@
         <v>22</v>
       </c>
       <c r="C35" s="21">
-        <f>IF(B35=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B35=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D35" s="21">
@@ -4666,7 +4666,7 @@
         <v>23</v>
       </c>
       <c r="C36" s="21">
-        <f>IF(B36=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B36=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D36" s="21">
@@ -4707,7 +4707,7 @@
         <v>24</v>
       </c>
       <c r="C37" s="21">
-        <f>IF(B37=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B37=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D37" s="21">
@@ -4748,7 +4748,7 @@
         <v>25</v>
       </c>
       <c r="C38" s="21">
-        <f>IF(B38=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B38=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D38" s="21">
@@ -4789,7 +4789,7 @@
         <v>26</v>
       </c>
       <c r="C39" s="21">
-        <f>IF(B39=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B39=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D39" s="21">
@@ -4830,7 +4830,7 @@
         <v>27</v>
       </c>
       <c r="C40" s="21">
-        <f>IF(B40=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B40=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D40" s="21">
@@ -4871,7 +4871,7 @@
         <v>28</v>
       </c>
       <c r="C41" s="21">
-        <f>IF(B41=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B41=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D41" s="21">
@@ -4912,7 +4912,7 @@
         <v>29</v>
       </c>
       <c r="C42" s="21">
-        <f>IF(B42=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B42=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D42" s="21">
@@ -4953,7 +4953,7 @@
         <v>30</v>
       </c>
       <c r="C43" s="21">
-        <f>IF(B43=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B43=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D43" s="21">
@@ -4994,7 +4994,7 @@
         <v>31</v>
       </c>
       <c r="C44" s="21">
-        <f>IF(B44=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B44=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D44" s="21">
@@ -5035,7 +5035,7 @@
         <v>32</v>
       </c>
       <c r="C45" s="21">
-        <f>IF(B45=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B45=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D45" s="21">
@@ -5076,7 +5076,7 @@
         <v>33</v>
       </c>
       <c r="C46" s="21">
-        <f>IF(B46=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B46=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D46" s="21">
@@ -5117,7 +5117,7 @@
         <v>34</v>
       </c>
       <c r="C47" s="21">
-        <f>IF(B47=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B47=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D47" s="21">
@@ -5158,7 +5158,7 @@
         <v>35</v>
       </c>
       <c r="C48" s="21">
-        <f>IF(B48=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B48=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D48" s="21">
@@ -5199,7 +5199,7 @@
         <v>36</v>
       </c>
       <c r="C49" s="21">
-        <f>IF(B49=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B49=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D49" s="21">
@@ -5240,7 +5240,7 @@
         <v>37</v>
       </c>
       <c r="C50" s="21">
-        <f>IF(B50=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B50=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D50" s="21">
@@ -5281,7 +5281,7 @@
         <v>38</v>
       </c>
       <c r="C51" s="21">
-        <f>IF(B51=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B51=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D51" s="21">
@@ -5322,7 +5322,7 @@
         <v>39</v>
       </c>
       <c r="C52" s="21">
-        <f>IF(B52=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B52=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D52" s="21">
@@ -5363,7 +5363,7 @@
         <v>40</v>
       </c>
       <c r="C53" s="21">
-        <f>IF(B53=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B53=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D53" s="21">
@@ -5404,7 +5404,7 @@
         <v>41</v>
       </c>
       <c r="C54" s="21">
-        <f>IF(B54=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B54=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D54" s="21">
@@ -5445,7 +5445,7 @@
         <v>42</v>
       </c>
       <c r="C55" s="21">
-        <f>IF(B55=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B55=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D55" s="21">
@@ -5486,7 +5486,7 @@
         <v>43</v>
       </c>
       <c r="C56" s="21">
-        <f>IF(B56=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B56=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D56" s="21">
@@ -5527,7 +5527,7 @@
         <v>44</v>
       </c>
       <c r="C57" s="21">
-        <f>IF(B57=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B57=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D57" s="21">
@@ -5568,7 +5568,7 @@
         <v>45</v>
       </c>
       <c r="C58" s="21">
-        <f>IF(B58=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B58=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D58" s="21">
@@ -5609,7 +5609,7 @@
         <v>46</v>
       </c>
       <c r="C59" s="21">
-        <f>IF(B59=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B59=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D59" s="21">
@@ -5650,7 +5650,7 @@
         <v>47</v>
       </c>
       <c r="C60" s="21">
-        <f>IF(B60=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B60=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D60" s="21">
@@ -5691,7 +5691,7 @@
         <v>48</v>
       </c>
       <c r="C61" s="21">
-        <f>IF(B61=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B61=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D61" s="21">
@@ -5732,7 +5732,7 @@
         <v>49</v>
       </c>
       <c r="C62" s="21">
-        <f>IF(B62=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B62=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D62" s="21">
@@ -5773,7 +5773,7 @@
         <v>50</v>
       </c>
       <c r="C63" s="21">
-        <f>IF(B63=0,'01_Supuestos'!$D$7,0)</f>
+        <f>IF(B63=0,'01_Supuestos'!$D$7*(1-'01_Supuestos'!$D$8),0)</f>
         <v/>
       </c>
       <c r="D63" s="21">

</xml_diff>